<commit_message>
docs: split daily reports into morning plan / evening result format
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ev2GcePRwbwZKfH9HbtDvV
</commit_message>
<xml_diff>
--- a/docs/scrap-highlight/스크랩하이라이트_DS도입_관리.xlsx
+++ b/docs/scrap-highlight/스크랩하이라이트_DS도입_관리.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="501" uniqueCount="356">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="382">
   <si>
     <t xml:space="preserve">스크랩 하이라이트 DS 도입 — 과제 관리</t>
   </si>
@@ -256,7 +256,7 @@
     <t xml:space="preserve">보고 루틴</t>
   </si>
   <si>
-    <t xml:space="preserve">매일 08:00 이한정 / 18:00 양진호 (정시 이전 게시, 텔레그램 전환 예정)</t>
+    <t xml:space="preserve">08:00 이한정 = 당일 진행계획 / 18:00 양진호 = 당일 진행결과 (계획·결과 섞지 않기, 08:00은 전날 작성·예약 발신)</t>
   </si>
   <si>
     <t xml:space="preserve">실무</t>
@@ -1202,6 +1202,112 @@
       </rPr>
       <t xml:space="preserve">시트</t>
     </r>
+  </si>
+  <si>
+    <t xml:space="preserve">A11</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ 18:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과 보고 분리 운영 — 퇴근 전 양진호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이한정 다음날 계획 합의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보고 예약 발신</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이한정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">양진호</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">매일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김기훈 부장 가이드</t>
   </si>
   <si>
     <t xml:space="preserve">기술 요건 체크리스트</t>
@@ -2936,10 +3042,804 @@
     <t xml:space="preserve">정기 보고: 팀장님 명의 공식 요청 필요, AX개발팀 실무방 개설, DX 도입일 미정(개발팀도 미확인), DS 보안 절차 확인 필요</t>
   </si>
   <si>
-    <t xml:space="preserve">정기 보고 로그</t>
-  </si>
-  <si>
-    <t xml:space="preserve">매일 08:00 이한정 / 18:00 양진호 · 정시 이전 게시 · 게시 후 원문을 한 행으로 붙여넣기</t>
+    <t xml:space="preserve">09:11</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보고 가이드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오전</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">당일 진행계획</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오후</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">=</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">당일 진행결과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">둘을 무 자르듯 분리</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재방송 방지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), 08:00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 전날 작성 후 예약 발신</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">정기 보고</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오전 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00 = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">당일 진행계획 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이한정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) / </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오후 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:00 = </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">당일 진행결과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">양진호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) · </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">김기훈 부장 가이드</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="9"/>
+        <color rgb="FF808080"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(10.27 09:11~09:16)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">보고 원칙</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오전 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 계획만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오후 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:00</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">은 결과만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획에 결과 섞지 않고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과에 내일 계획 섞지 않기 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">재방송</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">느낌 방지</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">① 전체 과정 중 현재 위치 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">어제까지 진척</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) ② </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오늘 할 협의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작업 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">담당</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) ③ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">막히는 지점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해결 필요 사항</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아침 계획 항목별로 ✅완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ 🟡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행중 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ ⛔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사유</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">조치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">). </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">속도 나서 추가로 간 것이 있으면 덧붙임</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">작성 요령</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:00~08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사이엔 진척이 없으므로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보고는 전날 퇴근 전 작성 → 예약 발신</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">두 사람이 퇴근 전 다음날 계획 미리 맞추기 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수건돌리기</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">연결</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오전 계획 항목 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">= </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오후 결과 항목이 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1:1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로 대응되도록 같은 번호 사용</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">유형</t>
   </si>
   <si>
     <t xml:space="preserve">보고자</t>
@@ -2954,7 +3854,54 @@
     <t xml:space="preserve">양식</t>
   </si>
   <si>
-    <t xml:space="preserve">직전 대비 변경점을 첫 줄에 / 지연은 원인+조치+필요 지원</t>
+    <t xml:space="preserve">08:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">계획</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현재 단계 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오늘 할 일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">막힌 점</t>
+    </r>
   </si>
   <si>
     <r>
@@ -3007,16 +3954,16 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">진행사항 보고드립니다</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. (MM.DD HH:00)
+      <t xml:space="preserve">금일 진행계획 보고드립니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. (MM.DD)
 1. </t>
     </r>
     <r>
@@ -3025,7 +3972,8 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">금일</t>
+      <t xml:space="preserve">현재 단계
+□ </t>
     </r>
     <r>
       <rPr>
@@ -3042,42 +3990,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">전일</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">진행사항
-□ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">핵심 한 줄</t>
+      <t xml:space="preserve">전체 과정 중 위치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">요청 → 샘플 테스트 → 세팅 → 병행 테스트 → 적용</t>
     </r>
     <r>
       <rPr>
@@ -3095,7 +4025,113 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">세부
+      <t xml:space="preserve">전일 진척</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있을 때만 한 줄</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">금일 진행계획
+① </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">협의</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">작업</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">담당</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">대상
+② 
+③ 
 </t>
     </r>
     <r>
@@ -3105,15 +4141,33 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">2. DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">진행 현황 </t>
+      <t xml:space="preserve">3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이슈 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">해결 필요
+□ </t>
     </r>
     <r>
       <rPr>
@@ -3130,61 +4184,24 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">변동 시</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)
-□
-3. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이슈 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">요청사항
-□ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">결재</t>
+      <t xml:space="preserve">막히는 지점</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">필요한 결재</t>
     </r>
     <r>
       <rPr>
@@ -3201,77 +4218,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">지원 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">지연 요인과 조치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)
-4. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">향후 계획
-□ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">다음 보고까지 할 일 — 담당</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">기한</t>
+      <t xml:space="preserve">지원</t>
     </r>
     <r>
       <rPr>
@@ -3302,7 +4249,445 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">공식 요청메일 필요, AX 실무방 개설, DX 도입일 미정(개발팀도 일정 미확인), DS 보안절차 확인 필요</t>
+    <t xml:space="preserve">18:00</t>
+  </si>
+  <si>
+    <t xml:space="preserve">결과</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아침 계획 항목별 결과 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 진척 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스크랩 하이라이트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도입</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&gt;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">금일 진행결과 보고드립니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. (MM.DD)
+1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획 대비 결과
+① </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">아침 계획 ①</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) — ✅</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ 🟡</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행중 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/ ⛔</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연
+   </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과 내용
+② 
+③ 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 진척 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있을 때만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+□ 
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연 사유 및 조치 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있을 때만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+□ 
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 상 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">현황</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">공식 요청메일 필요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, AX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">실무방 개설</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도입일 미정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개발팀도 미확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">), DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보안절차 확인 필요 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(※ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">원칙 확정 전 첫 보고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
   </si>
   <si>
     <r>
@@ -4260,7 +5645,870 @@
     </r>
   </si>
   <si>
-    <t xml:space="preserve">18:00</t>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초안</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">] </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오전 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">향후 계획</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' 4</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개 항목 기준</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&lt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스크랩 하이라이트 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도입</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">&gt;
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">금일 진행결과 보고드립니다</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. (10.27)
+※ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">오전 보고 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">향후 계획</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">항목 기준 — 결과 확인 후 채울 것
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획 대비 결과
+① 팀장님 명의 개발지원 요청 메일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">안재용 센터장</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">김상하 상무</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+   — [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+   - [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">초안 작성</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">상무님 검토</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">발송 여부</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+② DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스크랩</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">수기 하이라이트 샘플 준비
+   — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+   - [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목차 표지 포함 여부</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">묶음 기사 정보</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(set.txt) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">포함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+③ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개발팀 테스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">방문 일정 협의
+   — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">[</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+   - [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">우면동 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개발팀 방문 일자</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+④ </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보안</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">시스템 준비 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">방화벽</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·NASCA/DRM·GPT Tier 4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·PC)
+   — [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">완료</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">진행중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+   - [</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">담당 부서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">소요 기간 확인 결과</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+2. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">추가 진척 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있을 때만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+□ [DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도입일 확인 등</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">]
+3. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">지연 사유 및 조치 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">있을 때만</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)
+□ 
+- </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이 상 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">-</t>
+    </r>
   </si>
   <si>
     <r>
@@ -5008,7 +7256,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0%"/>
   </numFmts>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -5118,6 +7366,18 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FF1F3864"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b val="true"/>
+      <sz val="10"/>
       <name val="맑은 고딕"/>
       <family val="0"/>
       <charset val="1"/>
@@ -5126,8 +7386,9 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FF1F3864"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
   </fonts>
   <fills count="5">
@@ -5218,7 +7479,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="32">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -5299,11 +7560,43 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -5733,7 +8026,7 @@
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">COUNTIF(할일!$F$5:$F$300,"진행중")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">COUNTIF(할일!$F$5:$F$300,"완료")</f>
@@ -5745,7 +8038,7 @@
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">IFERROR(D14/SUM(B14:E14),0)</f>
-        <v>0.285714285714286</v>
+        <v>0.266666666666667</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5931,7 +8224,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="6"/>
@@ -6288,6 +8581,29 @@
       </c>
       <c r="G18" s="16" t="s">
         <v>116</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="16" t="s">
+        <v>117</v>
+      </c>
+      <c r="B19" s="20" t="s">
+        <v>93</v>
+      </c>
+      <c r="C19" s="16" t="s">
+        <v>118</v>
+      </c>
+      <c r="D19" s="20" t="s">
+        <v>119</v>
+      </c>
+      <c r="E19" s="20" t="s">
+        <v>120</v>
+      </c>
+      <c r="F19" s="20" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="20" t="s">
+        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -6338,12 +8654,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6351,13 +8667,13 @@
         <v>51</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>53</v>
@@ -6368,16 +8684,16 @@
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>72</v>
@@ -6388,16 +8704,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>128</v>
+        <v>133</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>72</v>
@@ -6408,16 +8724,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>129</v>
+        <v>134</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>130</v>
+        <v>135</v>
       </c>
       <c r="C7" s="16" t="s">
-        <v>131</v>
+        <v>136</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>132</v>
+        <v>137</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>66</v>
@@ -6428,16 +8744,16 @@
     </row>
     <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>133</v>
+        <v>138</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>134</v>
+        <v>139</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>135</v>
+        <v>140</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>136</v>
+        <v>141</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>66</v>
@@ -6448,16 +8764,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>137</v>
+        <v>142</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>138</v>
+        <v>143</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>139</v>
+        <v>144</v>
       </c>
       <c r="D9" s="16" t="s">
-        <v>140</v>
+        <v>145</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>66</v>
@@ -6468,16 +8784,16 @@
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>141</v>
+        <v>146</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>80</v>
       </c>
       <c r="C10" s="16" t="s">
-        <v>142</v>
+        <v>147</v>
       </c>
       <c r="D10" s="16" t="s">
-        <v>143</v>
+        <v>148</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>66</v>
@@ -6488,16 +8804,16 @@
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>144</v>
+        <v>149</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="16" t="s">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="D11" s="16" t="s">
-        <v>146</v>
+        <v>151</v>
       </c>
       <c r="E11" s="13" t="s">
         <v>66</v>
@@ -6508,16 +8824,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>147</v>
+        <v>152</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>80</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>148</v>
+        <v>153</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>149</v>
+        <v>154</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>66</v>
@@ -6528,22 +8844,22 @@
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
-        <v>150</v>
+        <v>155</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>151</v>
+        <v>156</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>152</v>
+        <v>157</v>
       </c>
       <c r="D13" s="16" t="s">
-        <v>153</v>
+        <v>158</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="F13" s="13" t="s">
-        <v>155</v>
+        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -6595,29 +8911,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>156</v>
+        <v>161</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>157</v>
+        <v>162</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>158</v>
+        <v>163</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>159</v>
+        <v>164</v>
       </c>
       <c r="C4" s="18" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="D4" s="18" t="s">
-        <v>161</v>
+        <v>166</v>
       </c>
       <c r="E4" s="19" t="s">
-        <v>162</v>
+        <v>167</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>55</v>
@@ -6625,17 +8941,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>163</v>
+        <v>168</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="C5" s="16" t="s">
-        <v>165</v>
-      </c>
-      <c r="D5" s="20"/>
+        <v>170</v>
+      </c>
+      <c r="D5" s="21"/>
       <c r="E5" s="16" t="s">
-        <v>166</v>
+        <v>171</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>18</v>
@@ -6643,15 +8959,15 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>167</v>
+        <v>172</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>168</v>
-      </c>
-      <c r="D6" s="20"/>
+        <v>173</v>
+      </c>
+      <c r="D6" s="21"/>
       <c r="E6" s="16" t="s">
         <v>74</v>
       </c>
@@ -6661,17 +8977,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>169</v>
+        <v>174</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>170</v>
+        <v>175</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>171</v>
-      </c>
-      <c r="D7" s="20"/>
+        <v>176</v>
+      </c>
+      <c r="D7" s="21"/>
       <c r="E7" s="16" t="s">
-        <v>172</v>
+        <v>177</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>18</v>
@@ -6679,17 +8995,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>173</v>
+        <v>178</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>154</v>
+        <v>159</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="20"/>
+      <c r="D8" s="21"/>
       <c r="E8" s="16" t="s">
-        <v>174</v>
+        <v>179</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>18</v>
@@ -6697,15 +9013,15 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>176</v>
+        <v>181</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>177</v>
-      </c>
-      <c r="D9" s="20"/>
+        <v>182</v>
+      </c>
+      <c r="D9" s="21"/>
       <c r="E9" s="16" t="s">
         <v>101</v>
       </c>
@@ -6715,16 +9031,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>178</v>
+        <v>183</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>179</v>
+        <v>184</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="D10" s="20" t="s">
-        <v>181</v>
+        <v>185</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>186</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="13" t="s">
@@ -6780,7 +9096,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>182</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -6788,291 +9104,291 @@
         <v>17</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>183</v>
+        <v>188</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>185</v>
+        <v>190</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>186</v>
+        <v>191</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>187</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>190</v>
+        <v>195</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>191</v>
+        <v>196</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>192</v>
+        <v>197</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>193</v>
+        <v>198</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>194</v>
+        <v>199</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>195</v>
+        <v>200</v>
       </c>
       <c r="F5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>196</v>
+        <v>201</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>198</v>
+        <v>203</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>200</v>
+        <v>205</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>201</v>
+        <v>206</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>202</v>
+        <v>207</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>203</v>
+        <v>208</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>204</v>
+        <v>209</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="13" t="s">
-        <v>205</v>
+        <v>210</v>
       </c>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>188</v>
+        <v>193</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="13" t="s">
-        <v>206</v>
+        <v>211</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="F11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="13" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>207</v>
+        <v>212</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="F14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>160</v>
+        <v>165</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="16" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="13" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="E18" s="16"/>
       <c r="F18" s="13" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="13" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -7091,7 +9407,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:D25"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -7102,108 +9418,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="13" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>252</v>
+        <v>257</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>256</v>
+        <v>261</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>251</v>
+        <v>256</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>258</v>
+        <v>263</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>259</v>
+        <v>264</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>260</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>262</v>
+        <v>267</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>264</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>261</v>
+        <v>266</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>265</v>
+        <v>270</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>253</v>
+        <v>258</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7212,10 +9528,10 @@
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="13" t="s">
-        <v>267</v>
+        <v>272</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>268</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7223,13 +9539,13 @@
         <v>107</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>269</v>
+        <v>274</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7237,13 +9553,13 @@
         <v>107</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>271</v>
+        <v>276</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>272</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7251,13 +9567,13 @@
         <v>107</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>273</v>
+        <v>278</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>274</v>
+        <v>279</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7265,13 +9581,13 @@
         <v>107</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>255</v>
+        <v>260</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>276</v>
+        <v>281</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7279,13 +9595,13 @@
         <v>107</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>277</v>
+        <v>282</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>278</v>
+        <v>283</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7293,13 +9609,13 @@
         <v>107</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>279</v>
+        <v>284</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>280</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7307,13 +9623,13 @@
         <v>107</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>281</v>
+        <v>286</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>282</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7321,13 +9637,13 @@
         <v>107</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>284</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7335,13 +9651,13 @@
         <v>107</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>283</v>
+        <v>288</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>285</v>
+        <v>290</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7349,13 +9665,13 @@
         <v>107</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>286</v>
+        <v>291</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>287</v>
+        <v>292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7363,13 +9679,13 @@
         <v>61</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>288</v>
+        <v>293</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>289</v>
+        <v>294</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>290</v>
+        <v>295</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7377,13 +9693,13 @@
         <v>61</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>291</v>
+        <v>296</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>263</v>
+        <v>268</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>292</v>
+        <v>297</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -7391,13 +9707,27 @@
         <v>61</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>293</v>
+        <v>298</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>294</v>
+        <v>299</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B25" s="16" t="s">
+        <v>300</v>
+      </c>
+      <c r="C25" s="20" t="s">
+        <v>99</v>
+      </c>
+      <c r="D25" s="20" t="s">
+        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -7416,87 +9746,206 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="7"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="40"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="90"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="2" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A2" s="17" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="19" t="s">
-        <v>244</v>
-      </c>
-      <c r="B4" s="19" t="s">
-        <v>245</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>297</v>
-      </c>
-      <c r="D4" s="19" t="s">
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="22" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="23" t="s">
+        <v>303</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="24" t="s">
+        <v>304</v>
+      </c>
+      <c r="B4" s="25"/>
+      <c r="C4" s="25"/>
+      <c r="D4" s="25"/>
+      <c r="E4" s="25"/>
+      <c r="F4" s="25"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="27" t="s">
+        <v>305</v>
+      </c>
+      <c r="C5" s="27"/>
+      <c r="D5" s="27"/>
+      <c r="E5" s="27"/>
+      <c r="F5" s="27"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="28" t="s">
+        <v>306</v>
+      </c>
+      <c r="B6" s="27" t="s">
+        <v>307</v>
+      </c>
+      <c r="C6" s="27"/>
+      <c r="D6" s="27"/>
+      <c r="E6" s="27"/>
+      <c r="F6" s="27"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="28" t="s">
+        <v>308</v>
+      </c>
+      <c r="B7" s="27" t="s">
+        <v>309</v>
+      </c>
+      <c r="C7" s="27"/>
+      <c r="D7" s="27"/>
+      <c r="E7" s="27"/>
+      <c r="F7" s="27"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="s">
+        <v>310</v>
+      </c>
+      <c r="B8" s="15" t="s">
+        <v>311</v>
+      </c>
+      <c r="C8" s="15"/>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15"/>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A9" s="26" t="s">
+        <v>312</v>
+      </c>
+      <c r="B9" s="27" t="s">
+        <v>313</v>
+      </c>
+      <c r="C9" s="27"/>
+      <c r="D9" s="27"/>
+      <c r="E9" s="27"/>
+      <c r="F9" s="27"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="24" t="s">
+        <v>249</v>
+      </c>
+      <c r="B11" s="24" t="s">
+        <v>250</v>
+      </c>
+      <c r="C11" s="24" t="s">
+        <v>314</v>
+      </c>
+      <c r="D11" s="24" t="s">
+        <v>315</v>
+      </c>
+      <c r="E11" s="24" t="s">
+        <v>316</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>317</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="B12" s="16" t="s">
+        <v>319</v>
+      </c>
+      <c r="C12" s="20" t="s">
+        <v>320</v>
+      </c>
+      <c r="D12" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="20" t="s">
+        <v>321</v>
+      </c>
+      <c r="F12" s="16" t="s">
+        <v>322</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="20" t="s">
+        <v>318</v>
+      </c>
+      <c r="B13" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="C13" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="D13" s="20" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="20" t="s">
+        <v>325</v>
+      </c>
+      <c r="F13" s="16" t="s">
+        <v>326</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A14" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B14" s="16" t="s">
         <v>298</v>
       </c>
-      <c r="E4" s="19" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="5" customFormat="false" ht="199.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="13" t="s">
-        <v>300</v>
-      </c>
-      <c r="B5" s="16"/>
-      <c r="C5" s="16"/>
-      <c r="D5" s="13" t="s">
-        <v>301</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="6" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="16" t="s">
+      <c r="C14" s="20" t="s">
+        <v>327</v>
+      </c>
+      <c r="D14" s="20" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="20" t="s">
+        <v>328</v>
+      </c>
+      <c r="F14" s="16" t="s">
+        <v>329</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A15" s="16" t="s">
         <v>61</v>
       </c>
-      <c r="B6" s="16" t="s">
-        <v>293</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>66</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>303</v>
-      </c>
-      <c r="E6" s="16" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="7" customFormat="false" ht="19.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="16" t="s">
-        <v>61</v>
-      </c>
-      <c r="B7" s="16" t="s">
-        <v>305</v>
-      </c>
-      <c r="C7" s="13" t="s">
+      <c r="B15" s="16" t="s">
+        <v>323</v>
+      </c>
+      <c r="C15" s="20" t="s">
+        <v>324</v>
+      </c>
+      <c r="D15" s="20" t="s">
         <v>72</v>
       </c>
-      <c r="D7" s="20"/>
-      <c r="E7" s="20"/>
+      <c r="E15" s="21" t="s">
+        <v>330</v>
+      </c>
+      <c r="F15" s="21" t="s">
+        <v>331</v>
+      </c>
     </row>
   </sheetData>
+  <mergeCells count="6">
+    <mergeCell ref="B4:F4"/>
+    <mergeCell ref="B5:F5"/>
+    <mergeCell ref="B6:F6"/>
+    <mergeCell ref="B7:F7"/>
+    <mergeCell ref="B8:F8"/>
+    <mergeCell ref="B9:F9"/>
+  </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
@@ -7520,53 +9969,53 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="21" t="s">
-        <v>306</v>
+      <c r="A1" s="29" t="s">
+        <v>332</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>307</v>
+        <v>333</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="22" t="s">
-        <v>308</v>
-      </c>
-      <c r="B4" s="20" t="s">
-        <v>309</v>
+      <c r="A4" s="30" t="s">
+        <v>334</v>
+      </c>
+      <c r="B4" s="21" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="22" t="s">
-        <v>310</v>
+      <c r="A5" s="30" t="s">
+        <v>336</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>311</v>
+        <v>337</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="22" t="s">
-        <v>312</v>
+      <c r="A6" s="30" t="s">
+        <v>338</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>313</v>
+        <v>339</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="22" t="s">
-        <v>314</v>
-      </c>
-      <c r="B7" s="20" t="s">
-        <v>315</v>
+      <c r="A7" s="30" t="s">
+        <v>340</v>
+      </c>
+      <c r="B7" s="21" t="s">
+        <v>341</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="420" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="22" t="s">
-        <v>316</v>
-      </c>
-      <c r="B8" s="23" t="s">
-        <v>317</v>
+      <c r="A8" s="30" t="s">
+        <v>342</v>
+      </c>
+      <c r="B8" s="31" t="s">
+        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -7595,205 +10044,205 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>318</v>
+        <v>344</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>319</v>
+        <v>345</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>320</v>
+        <v>346</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>322</v>
+        <v>348</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>323</v>
+        <v>349</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>324</v>
+        <v>350</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>325</v>
+        <v>351</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>326</v>
+        <v>352</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>327</v>
+        <v>353</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>328</v>
+        <v>354</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>329</v>
+        <v>355</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>330</v>
+        <v>356</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>331</v>
+        <v>357</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>332</v>
+        <v>358</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>333</v>
+        <v>359</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>334</v>
+        <v>360</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>335</v>
+        <v>361</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>336</v>
+        <v>362</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>337</v>
+        <v>363</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>338</v>
+        <v>364</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>339</v>
+        <v>365</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>340</v>
+        <v>366</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>341</v>
+        <v>367</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>342</v>
+        <v>368</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>343</v>
+        <v>369</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>321</v>
+        <v>347</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>344</v>
+        <v>370</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>345</v>
+        <v>371</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>347</v>
+        <v>373</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>348</v>
+        <v>374</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>349</v>
+        <v>375</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>350</v>
+        <v>376</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>351</v>
+        <v>377</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>266</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>352</v>
+        <v>378</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>353</v>
+        <v>379</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>346</v>
+        <v>372</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>354</v>
+        <v>380</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>355</v>
+        <v>381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: mark Telegram room transition as done
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ev2GcePRwbwZKfH9HbtDvV
</commit_message>
<xml_diff>
--- a/docs/scrap-highlight/스크랩하이라이트_DS도입_관리.xlsx
+++ b/docs/scrap-highlight/스크랩하이라이트_DS도입_관리.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="537" uniqueCount="382">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="381">
   <si>
     <t xml:space="preserve">스크랩 하이라이트 DS 도입 — 과제 관리</t>
   </si>
@@ -256,7 +256,7 @@
     <t xml:space="preserve">보고 루틴</t>
   </si>
   <si>
-    <t xml:space="preserve">08:00 이한정 = 당일 진행계획 / 18:00 양진호 = 당일 진행결과 (계획·결과 섞지 않기, 08:00은 전날 작성·예약 발신)</t>
+    <t xml:space="preserve">08:00 이한정 = 당일 진행계획 / 18:00 양진호 = 당일 진행결과 (텔레그램 방 · 계획·결과 섞지 않기, 08:00은 전날 작성·예약 발신)</t>
   </si>
   <si>
     <t xml:space="preserve">실무</t>
@@ -947,10 +947,10 @@
     <t xml:space="preserve">보고방 텔레그램 전환</t>
   </si>
   <si>
-    <t xml:space="preserve">이정섭 파트장(확인 필요)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기록 보존 목적</t>
+    <t xml:space="preserve">-</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10.27 텔레그램 방 개설 완료</t>
   </si>
   <si>
     <t xml:space="preserve">A9</t>
@@ -1277,13 +1277,106 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이한정</t>
+    <t xml:space="preserve">매일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김기훈 부장 가이드</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기술 요건 체크리스트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">출처: 김경수 파트장(전사 AX개발팀) Newspaper_Highlight.exe 선행조건 안내 / 차병석 부사장 안내메일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">분류</t>
+  </si>
+  <si>
+    <t xml:space="preserve">요건</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">확인 사항</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">입력</t>
+  </si>
+  <si>
+    <t xml:space="preserve">스크랩 PDF: 1p 목차 표지 포함 검토본</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스크랩에 목차 표지 있는지</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">양식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">단 구성</t>
     </r>
     <r>
       <rPr>
@@ -1300,33 +1393,138 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">양진호</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">매일</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김기훈 부장 가이드</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기술 요건 체크리스트</t>
-  </si>
-  <si>
-    <t xml:space="preserve">출처: 김경수 파트장(전사 AX개발팀) Newspaper_Highlight.exe 선행조건 안내 / 차병석 부사장 안내메일</t>
-  </si>
-  <si>
-    <t xml:space="preserve">분류</t>
-  </si>
-  <si>
-    <t xml:space="preserve">요건</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
+      <t xml:space="preserve">제목</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">/</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">본문 배치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차이</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">묶음 기사 정보 set.txt (예: - 헬릭스 투자 관련 : 5~6P)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">매일 새벽 스크랩 담당자 작성 프로세스 지정</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">PC</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Windows 11 64bit, RAM 16GB+, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">충분한 저장공간</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">스크랩 제작 PC 사양 확인 / 필요시 교체</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T4</t>
+  </si>
+  <si>
+    <t xml:space="preserve">계정</t>
+  </si>
+  <si>
+    <t xml:space="preserve">사내 외부 생성형 AI GPT Tier 4 권한 계정 (1회 300~350 크레딧)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">신청 절차·승인권자·소요기간, 비용 부담 주체</t>
+  </si>
+  <si>
+    <t xml:space="preserve">T5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SW</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">Codex CLI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">설치</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">로그인</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
         <rFont val="맑은 고딕"/>
         <family val="0"/>
         <charset val="1"/>
@@ -1335,23 +1533,43 @@
     </r>
     <r>
       <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">확인 사항</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T1</t>
-  </si>
-  <si>
-    <t xml:space="preserve">입력</t>
-  </si>
-  <si>
-    <t xml:space="preserve">스크랩 PDF: 1p 목차 표지 포함 검토본</t>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보안정책상 설치 허용 여부</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T6</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">OCR API </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">방화벽 등록</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: inference-doxa-newspaper-wogt.shuttle.sr-cloud.com</t>
+    </r>
   </si>
   <si>
     <r>
@@ -1369,24 +1587,178 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">스크랩에 목차 표지 있는지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">양식</t>
+      <t xml:space="preserve">방화벽 신청 부서</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">소요기간</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T7</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NASCA/DRM </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">신뢰 프로그램 등록 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(Newspaper_Highlight.exe)</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사업장 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">NASCA </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">담당</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">소요기간</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기사 텍스트 외부 AI(ChatGPT) 전송</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">정보보호</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·AI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">활용 정책 사전 검토 필요 여부</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">범위</t>
+  </si>
+  <si>
+    <t xml:space="preserve">특이 편집 기사 하이라이트 미적용</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">처럼 추가 학습 없이 수작업 처리 권고 </t>
     </r>
     <r>
       <rPr>
@@ -1403,405 +1775,6 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">단 구성</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">제목</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">본문 배치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">차이</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T2</t>
-  </si>
-  <si>
-    <t xml:space="preserve">묶음 기사 정보 set.txt (예: - 헬릭스 투자 관련 : 5~6P)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">매일 새벽 스크랩 담당자 작성 프로세스 지정</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">PC</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Windows 11 64bit, RAM 16GB+, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">충분한 저장공간</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">스크랩 제작 PC 사양 확인 / 필요시 교체</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T4</t>
-  </si>
-  <si>
-    <t xml:space="preserve">계정</t>
-  </si>
-  <si>
-    <t xml:space="preserve">사내 외부 생성형 AI GPT Tier 4 권한 계정 (1회 300~350 크레딧)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">신청 절차·승인권자·소요기간, 비용 부담 주체</t>
-  </si>
-  <si>
-    <t xml:space="preserve">T5</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SW</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">Codex CLI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">설치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로그인</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보안정책상 설치 허용 여부</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T6</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">OCR API </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">방화벽 등록</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: inference-doxa-newspaper-wogt.shuttle.sr-cloud.com</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">방화벽 신청 부서</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">소요기간</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T7</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NASCA/DRM </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">신뢰 프로그램 등록 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(Newspaper_Highlight.exe)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">사업장 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">NASCA </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">담당</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">소요기간</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기사 텍스트 외부 AI(ChatGPT) 전송</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">정보보호</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·AI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">활용 정책 사전 검토 필요 여부</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T9</t>
-  </si>
-  <si>
-    <t xml:space="preserve">범위</t>
-  </si>
-  <si>
-    <t xml:space="preserve">특이 편집 기사 하이라이트 미적용</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">처럼 추가 학습 없이 수작업 처리 권고 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">학습 시 샘플 </t>
     </r>
     <r>
@@ -1830,9 +1803,6 @@
       </rPr>
       <t xml:space="preserve">+)</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">-</t>
   </si>
   <si>
     <t xml:space="preserve">결정대기</t>
@@ -3045,81 +3015,108 @@
     <t xml:space="preserve">09:11</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보고 가이드</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오전</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">당일 진행계획</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오후</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">=</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">당일 진행결과</t>
+    <t xml:space="preserve">보고 가이드: 오전=당일 진행계획, 오후=당일 진행결과. 둘을 무 자르듯 분리(재방송 방지), 08:00은 전날 작성 후 예약 발신</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보고방 텔레그램 전환 완료</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정기 보고</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오전 08:00 = 당일 진행계획 (이한정) / 오후 18:00 = 당일 진행결과 (양진호) · 김기훈 부장 가이드(10.27 09:11~09:16)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보고 원칙</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오전 08:00은 계획만, 오후 18:00은 결과만. 계획에 결과 섞지 않고, 결과에 내일 계획 섞지 않기 → '재방송' 느낌 방지</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계획</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">① 전체 과정 중 현재 위치 (어제까지 진척) ② 오늘 할 협의·작업 (담당·대상) ③ 막히는 지점·해결 필요 사항</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">아침 계획 항목별로 ✅완료 / 🟡진행중 / ⛔지연(사유·조치). 속도 나서 추가로 간 것이 있으면 덧붙임</t>
+  </si>
+  <si>
+    <t xml:space="preserve">작성 요령</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">18:00~08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">사이엔 진척이 없으므로 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">08:00 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보고는 전날 퇴근 전 작성 → 예약 발신</t>
     </r>
     <r>
       <rPr>
@@ -3136,7 +3133,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">둘을 무 자르듯 분리</t>
+      <t xml:space="preserve">두 사람이 퇴근 전 다음날 계획 미리 맞추기 </t>
     </r>
     <r>
       <rPr>
@@ -3153,632 +3150,6 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">재방송 방지</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">), 08:00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 전날 작성 후 예약 발신</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">정기 보고</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오전 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">08:00 = </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">당일 진행계획 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이한정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) / </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오후 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">18:00 = </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">당일 진행결과 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">양진호</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">김기훈 부장 가이드</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="9"/>
-        <color rgb="FF808080"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(10.27 09:11~09:16)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">보고 원칙</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오전 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">08:00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 계획만</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오후 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">18:00</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">은 결과만</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">계획에 결과 섞지 않고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">결과에 내일 계획 섞지 않기 → </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">재방송</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">' </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">느낌 방지</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">08:00 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">계획</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">① 전체 과정 중 현재 위치 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">어제까지 진척</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) ② </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오늘 할 협의</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">작업 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">담당</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">대상</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) ③ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">막히는 지점</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">해결 필요 사항</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">18:00 </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">결과</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">아침 계획 항목별로 ✅완료 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ 🟡</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">진행중 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ ⛔</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">지연</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">사유</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">조치</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">). </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">속도 나서 추가로 간 것이 있으면 덧붙임</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">작성 요령</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">18:00~08:00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">사이엔 진척이 없으므로 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">08:00 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보고는 전날 퇴근 전 작성 → 예약 발신</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">두 사람이 퇴근 전 다음날 계획 미리 맞추기 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
       <t xml:space="preserve">수건돌리기</t>
     </r>
     <r>
@@ -3795,48 +3166,7 @@
     <t xml:space="preserve">연결</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오전 계획 항목 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">= </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오후 결과 항목이 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1:1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">로 대응되도록 같은 번호 사용</t>
-    </r>
+    <t xml:space="preserve">오전 계획 항목 = 오후 결과 항목이 1:1로 대응되도록 같은 번호 사용</t>
   </si>
   <si>
     <t xml:space="preserve">유형</t>
@@ -3860,48 +3190,7 @@
     <t xml:space="preserve">계획</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">현재 단계 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">오늘 할 일 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">막힌 점</t>
-    </r>
+    <t xml:space="preserve">현재 단계 / 오늘 할 일 / 막힌 점</t>
   </si>
   <si>
     <r>
@@ -4255,48 +3544,7 @@
     <t xml:space="preserve">결과</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">아침 계획 항목별 결과 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">추가 진척 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">/ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">지연</t>
-    </r>
+    <t xml:space="preserve">아침 계획 항목별 결과 / 추가 진척 / 지연</t>
   </si>
   <si>
     <r>
@@ -4559,135 +3807,10 @@
     </r>
   </si>
   <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">현황</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">계획</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">공식 요청메일 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, AX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">실무방 개설</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도입일 미정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개발팀도 미확인</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">), DS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보안절차 확인 필요 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(※ </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">원칙 확정 전 첫 보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
+    <t xml:space="preserve">현황·계획</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공식 요청메일 필요, AX 실무방 개설, DX 도입일 미정(개발팀도 미확인), DS 보안절차 확인 필요 (※ 원칙 확정 전 첫 보고)</t>
   </si>
   <si>
     <r>
@@ -7364,10 +6487,10 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="14"/>
-      <color rgb="FF1F3864"/>
-      <name val="WenQuanYi Zen Hei"/>
-      <family val="2"/>
+      <sz val="10"/>
+      <name val="맑은 고딕"/>
+      <family val="0"/>
+      <charset val="1"/>
     </font>
     <font>
       <b val="true"/>
@@ -7377,7 +6500,8 @@
     </font>
     <font>
       <b val="true"/>
-      <sz val="10"/>
+      <sz val="14"/>
+      <color rgb="FF1F3864"/>
       <name val="맑은 고딕"/>
       <family val="0"/>
       <charset val="1"/>
@@ -7386,9 +6510,8 @@
       <b val="true"/>
       <sz val="14"/>
       <color rgb="FF1F3864"/>
-      <name val="맑은 고딕"/>
-      <family val="0"/>
-      <charset val="1"/>
+      <name val="WenQuanYi Zen Hei"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -7479,7 +6602,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="28">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7560,23 +6683,11 @@
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
     <xf numFmtId="164" fontId="8" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="15" fillId="3" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -7584,19 +6695,15 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="17" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="2" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="16" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="18" fillId="2" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
-      <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="164" fontId="19" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="18" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8022,7 +7129,7 @@
       </c>
       <c r="B14" s="9" t="n">
         <f aca="false">COUNTIF(할일!$F$5:$F$300,"미착수")</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C14" s="9" t="n">
         <f aca="false">COUNTIF(할일!$F$5:$F$300,"진행중")</f>
@@ -8030,7 +7137,7 @@
       </c>
       <c r="D14" s="9" t="n">
         <f aca="false">COUNTIF(할일!$F$5:$F$300,"완료")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E14" s="9" t="n">
         <f aca="false">COUNTIF(할일!$F$5:$F$300,"블로킹")</f>
@@ -8038,7 +7145,7 @@
       </c>
       <c r="F14" s="10" t="n">
         <f aca="false">IFERROR(D14/SUM(B14:E14),0)</f>
-        <v>0.266666666666667</v>
+        <v>0.333333333333333</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8447,7 +7554,7 @@
         <v>61</v>
       </c>
       <c r="F12" s="13" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G12" s="13" t="s">
         <v>96</v>
@@ -8583,27 +7690,27 @@
         <v>116</v>
       </c>
     </row>
-    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+    <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
         <v>117</v>
       </c>
-      <c r="B19" s="20" t="s">
+      <c r="B19" s="13" t="s">
         <v>93</v>
       </c>
       <c r="C19" s="16" t="s">
         <v>118</v>
       </c>
-      <c r="D19" s="20" t="s">
+      <c r="D19" s="13" t="s">
+        <v>60</v>
+      </c>
+      <c r="E19" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="E19" s="20" t="s">
+      <c r="F19" s="13" t="s">
+        <v>19</v>
+      </c>
+      <c r="G19" s="13" t="s">
         <v>120</v>
-      </c>
-      <c r="F19" s="20" t="s">
-        <v>19</v>
-      </c>
-      <c r="G19" s="20" t="s">
-        <v>121</v>
       </c>
     </row>
   </sheetData>
@@ -8654,12 +7761,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8667,13 +7774,13 @@
         <v>51</v>
       </c>
       <c r="B4" s="19" t="s">
+        <v>123</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>124</v>
       </c>
-      <c r="C4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>125</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>126</v>
       </c>
       <c r="E4" s="19" t="s">
         <v>53</v>
@@ -8684,16 +7791,16 @@
     </row>
     <row r="5" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
+        <v>126</v>
+      </c>
+      <c r="B5" s="13" t="s">
         <v>127</v>
       </c>
-      <c r="B5" s="13" t="s">
+      <c r="C5" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="D5" s="16" t="s">
         <v>129</v>
-      </c>
-      <c r="D5" s="16" t="s">
-        <v>130</v>
       </c>
       <c r="E5" s="13" t="s">
         <v>72</v>
@@ -8704,16 +7811,16 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
+        <v>130</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>131</v>
       </c>
-      <c r="B6" s="13" t="s">
-        <v>128</v>
-      </c>
-      <c r="C6" s="13" t="s">
+      <c r="D6" s="13" t="s">
         <v>132</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>133</v>
       </c>
       <c r="E6" s="13" t="s">
         <v>72</v>
@@ -8724,16 +7831,16 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
+        <v>133</v>
+      </c>
+      <c r="B7" s="16" t="s">
         <v>134</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="C7" s="16" t="s">
         <v>135</v>
       </c>
-      <c r="C7" s="16" t="s">
+      <c r="D7" s="13" t="s">
         <v>136</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>137</v>
       </c>
       <c r="E7" s="13" t="s">
         <v>66</v>
@@ -8744,16 +7851,16 @@
     </row>
     <row r="8" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
+        <v>137</v>
+      </c>
+      <c r="B8" s="13" t="s">
         <v>138</v>
       </c>
-      <c r="B8" s="13" t="s">
+      <c r="C8" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="C8" s="13" t="s">
+      <c r="D8" s="13" t="s">
         <v>140</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>141</v>
       </c>
       <c r="E8" s="13" t="s">
         <v>66</v>
@@ -8764,16 +7871,16 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
+        <v>141</v>
+      </c>
+      <c r="B9" s="16" t="s">
         <v>142</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="C9" s="16" t="s">
         <v>143</v>
       </c>
-      <c r="C9" s="16" t="s">
+      <c r="D9" s="16" t="s">
         <v>144</v>
-      </c>
-      <c r="D9" s="16" t="s">
-        <v>145</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>66</v>
@@ -8784,16 +7891,16 @@
     </row>
     <row r="10" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>80</v>
       </c>
       <c r="C10" s="16" t="s">
+        <v>146</v>
+      </c>
+      <c r="D10" s="16" t="s">
         <v>147</v>
-      </c>
-      <c r="D10" s="16" t="s">
-        <v>148</v>
       </c>
       <c r="E10" s="13" t="s">
         <v>66</v>
@@ -8804,16 +7911,16 @@
     </row>
     <row r="11" customFormat="false" ht="25.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="16" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B11" s="13" t="s">
         <v>80</v>
       </c>
       <c r="C11" s="16" t="s">
+        <v>149</v>
+      </c>
+      <c r="D11" s="16" t="s">
         <v>150</v>
-      </c>
-      <c r="D11" s="16" t="s">
-        <v>151</v>
       </c>
       <c r="E11" s="13" t="s">
         <v>66</v>
@@ -8824,16 +7931,16 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="16" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B12" s="13" t="s">
         <v>80</v>
       </c>
       <c r="C12" s="13" t="s">
+        <v>152</v>
+      </c>
+      <c r="D12" s="16" t="s">
         <v>153</v>
-      </c>
-      <c r="D12" s="16" t="s">
-        <v>154</v>
       </c>
       <c r="E12" s="13" t="s">
         <v>66</v>
@@ -8844,22 +7951,22 @@
     </row>
     <row r="13" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="16" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" s="13" t="s">
         <v>155</v>
       </c>
-      <c r="B13" s="13" t="s">
+      <c r="C13" s="13" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="D13" s="16" t="s">
         <v>157</v>
       </c>
-      <c r="D13" s="16" t="s">
+      <c r="E13" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="F13" s="13" t="s">
         <v>158</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>159</v>
-      </c>
-      <c r="F13" s="13" t="s">
-        <v>160</v>
       </c>
     </row>
   </sheetData>
@@ -8911,29 +8018,29 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
+        <v>161</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>162</v>
+      </c>
+      <c r="C4" s="18" t="s">
         <v>163</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="D4" s="18" t="s">
         <v>164</v>
       </c>
-      <c r="C4" s="18" t="s">
+      <c r="E4" s="19" t="s">
         <v>165</v>
-      </c>
-      <c r="D4" s="18" t="s">
-        <v>166</v>
-      </c>
-      <c r="E4" s="19" t="s">
-        <v>167</v>
       </c>
       <c r="F4" s="19" t="s">
         <v>55</v>
@@ -8941,17 +8048,17 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
+        <v>166</v>
+      </c>
+      <c r="B5" s="16" t="s">
+        <v>167</v>
+      </c>
+      <c r="C5" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="B5" s="16" t="s">
+      <c r="D5" s="20"/>
+      <c r="E5" s="16" t="s">
         <v>169</v>
-      </c>
-      <c r="C5" s="16" t="s">
-        <v>170</v>
-      </c>
-      <c r="D5" s="21"/>
-      <c r="E5" s="16" t="s">
-        <v>171</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>18</v>
@@ -8959,15 +8066,15 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>159</v>
+        <v>95</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>173</v>
-      </c>
-      <c r="D6" s="21"/>
+        <v>171</v>
+      </c>
+      <c r="D6" s="20"/>
       <c r="E6" s="16" t="s">
         <v>74</v>
       </c>
@@ -8977,17 +8084,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
+        <v>172</v>
+      </c>
+      <c r="B7" s="16" t="s">
+        <v>173</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>174</v>
       </c>
-      <c r="B7" s="16" t="s">
+      <c r="D7" s="20"/>
+      <c r="E7" s="16" t="s">
         <v>175</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>176</v>
-      </c>
-      <c r="D7" s="21"/>
-      <c r="E7" s="16" t="s">
-        <v>177</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>18</v>
@@ -8995,17 +8102,17 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>159</v>
+        <v>95</v>
       </c>
       <c r="C8" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="21"/>
+      <c r="D8" s="20"/>
       <c r="E8" s="16" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>18</v>
@@ -9013,15 +8120,15 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
+        <v>178</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>179</v>
+      </c>
+      <c r="C9" s="16" t="s">
         <v>180</v>
       </c>
-      <c r="B9" s="16" t="s">
-        <v>181</v>
-      </c>
-      <c r="C9" s="16" t="s">
-        <v>182</v>
-      </c>
-      <c r="D9" s="21"/>
+      <c r="D9" s="20"/>
       <c r="E9" s="16" t="s">
         <v>101</v>
       </c>
@@ -9031,16 +8138,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" s="16" t="s">
+        <v>182</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>183</v>
       </c>
-      <c r="B10" s="16" t="s">
+      <c r="D10" s="20" t="s">
         <v>184</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>185</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>186</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="13" t="s">
@@ -9096,7 +8203,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9104,291 +8211,291 @@
         <v>17</v>
       </c>
       <c r="B3" s="19" t="s">
+        <v>186</v>
+      </c>
+      <c r="C3" s="19" t="s">
+        <v>187</v>
+      </c>
+      <c r="D3" s="19" t="s">
         <v>188</v>
       </c>
-      <c r="C3" s="19" t="s">
+      <c r="E3" s="19" t="s">
         <v>189</v>
       </c>
-      <c r="D3" s="19" t="s">
+      <c r="F3" s="19" t="s">
         <v>190</v>
-      </c>
-      <c r="E3" s="19" t="s">
-        <v>191</v>
-      </c>
-      <c r="F3" s="19" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
+        <v>191</v>
+      </c>
+      <c r="B4" s="16" t="s">
+        <v>192</v>
+      </c>
+      <c r="C4" s="13" t="s">
         <v>193</v>
       </c>
-      <c r="B4" s="16" t="s">
+      <c r="D4" s="13" t="s">
         <v>194</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>195</v>
-      </c>
-      <c r="D4" s="13" t="s">
-        <v>196</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>195</v>
+      </c>
+      <c r="C5" s="13" t="s">
+        <v>196</v>
+      </c>
+      <c r="D5" s="13" t="s">
         <v>197</v>
       </c>
-      <c r="C5" s="13" t="s">
+      <c r="E5" s="16" t="s">
         <v>198</v>
-      </c>
-      <c r="D5" s="13" t="s">
-        <v>199</v>
-      </c>
-      <c r="E5" s="16" t="s">
-        <v>200</v>
       </c>
       <c r="F5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B6" s="13" t="s">
+        <v>199</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>200</v>
+      </c>
+      <c r="D6" s="13" t="s">
         <v>201</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>202</v>
-      </c>
-      <c r="D6" s="13" t="s">
-        <v>203</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B8" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>205</v>
+      </c>
+      <c r="D8" s="13" t="s">
         <v>206</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>207</v>
-      </c>
-      <c r="D8" s="13" t="s">
-        <v>208</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="13" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="13" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
+        <v>210</v>
+      </c>
+      <c r="B11" s="13" t="s">
+        <v>211</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>212</v>
       </c>
-      <c r="B11" s="13" t="s">
+      <c r="D11" s="13" t="s">
         <v>213</v>
       </c>
-      <c r="C11" s="13" t="s">
+      <c r="E11" s="16" t="s">
         <v>214</v>
-      </c>
-      <c r="D11" s="13" t="s">
-        <v>215</v>
-      </c>
-      <c r="E11" s="16" t="s">
-        <v>216</v>
       </c>
       <c r="F11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="13" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B13" s="13" t="s">
+        <v>217</v>
+      </c>
+      <c r="C13" s="13" t="s">
+        <v>218</v>
+      </c>
+      <c r="D13" s="13" t="s">
         <v>219</v>
       </c>
-      <c r="C13" s="13" t="s">
+      <c r="E13" s="16" t="s">
         <v>220</v>
       </c>
-      <c r="D13" s="13" t="s">
+      <c r="F13" s="16" t="s">
         <v>221</v>
-      </c>
-      <c r="E13" s="16" t="s">
-        <v>222</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>223</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="16" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B14" s="13" t="s">
+        <v>222</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>223</v>
+      </c>
+      <c r="D14" s="16" t="s">
         <v>224</v>
       </c>
-      <c r="C14" s="13" t="s">
+      <c r="E14" s="16" t="s">
         <v>225</v>
-      </c>
-      <c r="D14" s="16" t="s">
-        <v>226</v>
-      </c>
-      <c r="E14" s="16" t="s">
-        <v>227</v>
       </c>
       <c r="F14" s="16"/>
     </row>
     <row r="15" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="16" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="B15" s="13" t="s">
+        <v>226</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>227</v>
+      </c>
+      <c r="D15" s="16" t="s">
         <v>228</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>229</v>
-      </c>
-      <c r="D15" s="16" t="s">
-        <v>230</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="16" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
+        <v>230</v>
+      </c>
+      <c r="B16" s="13" t="s">
+        <v>231</v>
+      </c>
+      <c r="C16" s="13" t="s">
         <v>232</v>
       </c>
-      <c r="B16" s="13" t="s">
+      <c r="D16" s="13" t="s">
         <v>233</v>
       </c>
-      <c r="C16" s="13" t="s">
+      <c r="E16" s="16" t="s">
         <v>234</v>
       </c>
-      <c r="D16" s="13" t="s">
+      <c r="F16" s="13" t="s">
         <v>235</v>
-      </c>
-      <c r="E16" s="16" t="s">
-        <v>236</v>
-      </c>
-      <c r="F16" s="13" t="s">
-        <v>237</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B17" s="13" t="s">
+        <v>236</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>237</v>
+      </c>
+      <c r="D17" s="13" t="s">
         <v>238</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>239</v>
-      </c>
-      <c r="D17" s="13" t="s">
-        <v>240</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="13" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B18" s="13" t="s">
+        <v>239</v>
+      </c>
+      <c r="C18" s="13" t="s">
+        <v>240</v>
+      </c>
+      <c r="D18" s="13" t="s">
         <v>241</v>
-      </c>
-      <c r="C18" s="13" t="s">
-        <v>242</v>
-      </c>
-      <c r="D18" s="13" t="s">
-        <v>243</v>
       </c>
       <c r="E18" s="16"/>
       <c r="F18" s="13" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>245</v>
+        <v>243</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>246</v>
+        <v>244</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="13" t="s">
-        <v>244</v>
+        <v>242</v>
       </c>
     </row>
   </sheetData>
@@ -9407,7 +8514,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -9418,108 +8525,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>247</v>
+        <v>245</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>248</v>
+        <v>246</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
+        <v>247</v>
+      </c>
+      <c r="B4" s="19" t="s">
+        <v>248</v>
+      </c>
+      <c r="C4" s="19" t="s">
         <v>249</v>
       </c>
-      <c r="B4" s="19" t="s">
+      <c r="D4" s="19" t="s">
         <v>250</v>
-      </c>
-      <c r="C4" s="19" t="s">
-        <v>251</v>
-      </c>
-      <c r="D4" s="19" t="s">
-        <v>252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="13" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
+        <v>254</v>
+      </c>
+      <c r="B6" s="16" t="s">
+        <v>255</v>
+      </c>
+      <c r="C6" s="13" t="s">
         <v>256</v>
       </c>
-      <c r="B6" s="16" t="s">
+      <c r="D6" s="16" t="s">
         <v>257</v>
-      </c>
-      <c r="C6" s="13" t="s">
-        <v>258</v>
-      </c>
-      <c r="D6" s="16" t="s">
-        <v>259</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B7" s="16" t="s">
+        <v>258</v>
+      </c>
+      <c r="C7" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="D7" s="13" t="s">
         <v>260</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>261</v>
-      </c>
-      <c r="D7" s="13" t="s">
-        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B8" s="16" t="s">
+        <v>261</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>262</v>
+      </c>
+      <c r="D8" s="16" t="s">
         <v>263</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>264</v>
-      </c>
-      <c r="D8" s="16" t="s">
-        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
+        <v>264</v>
+      </c>
+      <c r="B9" s="16" t="s">
+        <v>265</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>266</v>
       </c>
-      <c r="B9" s="16" t="s">
+      <c r="D9" s="13" t="s">
         <v>267</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="D9" s="13" t="s">
-        <v>269</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9528,10 +8635,10 @@
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="13" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9539,13 +8646,13 @@
         <v>107</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9553,13 +8660,13 @@
         <v>107</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9567,13 +8674,13 @@
         <v>107</v>
       </c>
       <c r="B14" s="16" t="s">
+        <v>276</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>277</v>
+      </c>
+      <c r="D14" s="13" t="s">
         <v>278</v>
-      </c>
-      <c r="C14" s="13" t="s">
-        <v>279</v>
-      </c>
-      <c r="D14" s="13" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9581,13 +8688,13 @@
         <v>107</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9595,13 +8702,13 @@
         <v>107</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9609,13 +8716,13 @@
         <v>107</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9623,13 +8730,13 @@
         <v>107</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9637,13 +8744,13 @@
         <v>107</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9651,13 +8758,13 @@
         <v>107</v>
       </c>
       <c r="B20" s="16" t="s">
+        <v>286</v>
+      </c>
+      <c r="C20" s="13" t="s">
+        <v>266</v>
+      </c>
+      <c r="D20" s="13" t="s">
         <v>288</v>
-      </c>
-      <c r="C20" s="13" t="s">
-        <v>268</v>
-      </c>
-      <c r="D20" s="13" t="s">
-        <v>290</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9665,13 +8772,13 @@
         <v>107</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9679,13 +8786,13 @@
         <v>61</v>
       </c>
       <c r="B22" s="16" t="s">
+        <v>291</v>
+      </c>
+      <c r="C22" s="13" t="s">
+        <v>292</v>
+      </c>
+      <c r="D22" s="16" t="s">
         <v>293</v>
-      </c>
-      <c r="C22" s="13" t="s">
-        <v>294</v>
-      </c>
-      <c r="D22" s="16" t="s">
-        <v>295</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9693,13 +8800,13 @@
         <v>61</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9707,27 +8814,39 @@
         <v>61</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>297</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A25" s="16" t="s">
         <v>61</v>
       </c>
       <c r="B25" s="16" t="s">
+        <v>298</v>
+      </c>
+      <c r="C25" s="13" t="s">
+        <v>99</v>
+      </c>
+      <c r="D25" s="13" t="s">
+        <v>299</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D26" s="21" t="s">
         <v>300</v>
-      </c>
-      <c r="C25" s="20" t="s">
-        <v>99</v>
-      </c>
-      <c r="D25" s="20" t="s">
-        <v>301</v>
       </c>
     </row>
   </sheetData>
@@ -9749,76 +8868,76 @@
   <dimension ref="A1:F15"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="12"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="8"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="10"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="9"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="36"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="70"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="8"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="10"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="36"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="70"/>
   </cols>
   <sheetData>
-    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A1" s="22" t="s">
+    <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A1" s="2" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="17" t="s">
         <v>302</v>
       </c>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="23" t="s">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
         <v>303</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A4" s="24" t="s">
+      <c r="B4" s="22"/>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+      <c r="E4" s="22"/>
+      <c r="F4" s="22"/>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="23" t="s">
+        <v>17</v>
+      </c>
+      <c r="B5" s="14" t="s">
         <v>304</v>
       </c>
-      <c r="B4" s="25"/>
-      <c r="C4" s="25"/>
-      <c r="D4" s="25"/>
-      <c r="E4" s="25"/>
-      <c r="F4" s="25"/>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="B5" s="27" t="s">
+      <c r="C5" s="14"/>
+      <c r="D5" s="14"/>
+      <c r="E5" s="14"/>
+      <c r="F5" s="14"/>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="24" t="s">
         <v>305</v>
       </c>
-      <c r="C5" s="27"/>
-      <c r="D5" s="27"/>
-      <c r="E5" s="27"/>
-      <c r="F5" s="27"/>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="28" t="s">
+      <c r="B6" s="14" t="s">
         <v>306</v>
       </c>
-      <c r="B6" s="27" t="s">
+      <c r="C6" s="14"/>
+      <c r="D6" s="14"/>
+      <c r="E6" s="14"/>
+      <c r="F6" s="14"/>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="24" t="s">
         <v>307</v>
       </c>
-      <c r="C6" s="27"/>
-      <c r="D6" s="27"/>
-      <c r="E6" s="27"/>
-      <c r="F6" s="27"/>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="28" t="s">
+      <c r="B7" s="14" t="s">
         <v>308</v>
       </c>
-      <c r="B7" s="27" t="s">
+      <c r="C7" s="14"/>
+      <c r="D7" s="14"/>
+      <c r="E7" s="14"/>
+      <c r="F7" s="14"/>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="23" t="s">
         <v>309</v>
       </c>
-      <c r="C7" s="27"/>
-      <c r="D7" s="27"/>
-      <c r="E7" s="27"/>
-      <c r="F7" s="27"/>
-    </row>
-    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="26" t="s">
+      <c r="B8" s="15" t="s">
         <v>310</v>
-      </c>
-      <c r="B8" s="15" t="s">
-        <v>311</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
@@ -9826,75 +8945,75 @@
       <c r="F8" s="15"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A9" s="26" t="s">
+      <c r="A9" s="23" t="s">
+        <v>311</v>
+      </c>
+      <c r="B9" s="14" t="s">
         <v>312</v>
       </c>
-      <c r="B9" s="27" t="s">
+      <c r="C9" s="14"/>
+      <c r="D9" s="14"/>
+      <c r="E9" s="14"/>
+      <c r="F9" s="14"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A11" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>248</v>
+      </c>
+      <c r="C11" s="11" t="s">
         <v>313</v>
       </c>
-      <c r="C9" s="27"/>
-      <c r="D9" s="27"/>
-      <c r="E9" s="27"/>
-      <c r="F9" s="27"/>
-    </row>
-    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A11" s="24" t="s">
-        <v>249</v>
-      </c>
-      <c r="B11" s="24" t="s">
-        <v>250</v>
-      </c>
-      <c r="C11" s="24" t="s">
+      <c r="D11" s="11" t="s">
         <v>314</v>
       </c>
-      <c r="D11" s="24" t="s">
+      <c r="E11" s="11" t="s">
         <v>315</v>
       </c>
-      <c r="E11" s="24" t="s">
+      <c r="F11" s="11" t="s">
         <v>316</v>
       </c>
-      <c r="F11" s="24" t="s">
+    </row>
+    <row r="12" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A12" s="13" t="s">
         <v>317</v>
       </c>
-    </row>
-    <row r="12" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A12" s="20" t="s">
+      <c r="B12" s="16" t="s">
         <v>318</v>
       </c>
-      <c r="B12" s="16" t="s">
+      <c r="C12" s="13" t="s">
         <v>319</v>
       </c>
-      <c r="C12" s="20" t="s">
+      <c r="D12" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E12" s="13" t="s">
         <v>320</v>
       </c>
-      <c r="D12" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="E12" s="20" t="s">
+      <c r="F12" s="16" t="s">
         <v>321</v>
       </c>
-      <c r="F12" s="16" t="s">
+    </row>
+    <row r="13" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A13" s="13" t="s">
+        <v>317</v>
+      </c>
+      <c r="B13" s="16" t="s">
         <v>322</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A13" s="20" t="s">
-        <v>318</v>
-      </c>
-      <c r="B13" s="16" t="s">
+      <c r="C13" s="13" t="s">
         <v>323</v>
       </c>
-      <c r="C13" s="20" t="s">
+      <c r="D13" s="13" t="s">
+        <v>72</v>
+      </c>
+      <c r="E13" s="13" t="s">
         <v>324</v>
       </c>
-      <c r="D13" s="20" t="s">
-        <v>72</v>
-      </c>
-      <c r="E13" s="20" t="s">
+      <c r="F13" s="16" t="s">
         <v>325</v>
-      </c>
-      <c r="F13" s="16" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9902,19 +9021,19 @@
         <v>61</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>298</v>
-      </c>
-      <c r="C14" s="20" t="s">
+        <v>296</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>326</v>
+      </c>
+      <c r="D14" s="13" t="s">
+        <v>66</v>
+      </c>
+      <c r="E14" s="13" t="s">
         <v>327</v>
       </c>
-      <c r="D14" s="20" t="s">
-        <v>66</v>
-      </c>
-      <c r="E14" s="20" t="s">
+      <c r="F14" s="16" t="s">
         <v>328</v>
-      </c>
-      <c r="F14" s="16" t="s">
-        <v>329</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9922,19 +9041,19 @@
         <v>61</v>
       </c>
       <c r="B15" s="16" t="s">
+        <v>322</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>323</v>
       </c>
-      <c r="C15" s="20" t="s">
-        <v>324</v>
-      </c>
-      <c r="D15" s="20" t="s">
+      <c r="D15" s="13" t="s">
         <v>72</v>
       </c>
-      <c r="E15" s="21" t="s">
+      <c r="E15" s="20" t="s">
+        <v>329</v>
+      </c>
+      <c r="F15" s="20" t="s">
         <v>330</v>
-      </c>
-      <c r="F15" s="21" t="s">
-        <v>331</v>
       </c>
     </row>
   </sheetData>
@@ -9969,53 +9088,53 @@
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A1" s="29" t="s">
-        <v>332</v>
+      <c r="A1" s="25" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
+        <v>332</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="26" t="s">
         <v>333</v>
       </c>
-    </row>
-    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A4" s="30" t="s">
+      <c r="B4" s="20" t="s">
         <v>334</v>
       </c>
-      <c r="B4" s="21" t="s">
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A5" s="26" t="s">
         <v>335</v>
       </c>
-    </row>
-    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A5" s="30" t="s">
+      <c r="B5" s="16" t="s">
         <v>336</v>
       </c>
-      <c r="B5" s="16" t="s">
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A6" s="26" t="s">
         <v>337</v>
       </c>
-    </row>
-    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A6" s="30" t="s">
+      <c r="B6" s="16" t="s">
         <v>338</v>
       </c>
-      <c r="B6" s="16" t="s">
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A7" s="26" t="s">
         <v>339</v>
       </c>
-    </row>
-    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A7" s="30" t="s">
+      <c r="B7" s="20" t="s">
         <v>340</v>
       </c>
-      <c r="B7" s="21" t="s">
+    </row>
+    <row r="8" customFormat="false" ht="420" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A8" s="26" t="s">
         <v>341</v>
       </c>
-    </row>
-    <row r="8" customFormat="false" ht="420" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="A8" s="30" t="s">
+      <c r="B8" s="27" t="s">
         <v>342</v>
-      </c>
-      <c r="B8" s="31" t="s">
-        <v>343</v>
       </c>
     </row>
   </sheetData>
@@ -10044,205 +9163,205 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>344</v>
+        <v>343</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
+        <v>344</v>
+      </c>
+      <c r="B3" s="19" t="s">
         <v>345</v>
       </c>
-      <c r="B3" s="19" t="s">
-        <v>346</v>
-      </c>
       <c r="C3" s="19" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
+        <v>346</v>
+      </c>
+      <c r="B4" s="13" t="s">
         <v>347</v>
       </c>
-      <c r="B4" s="13" t="s">
+      <c r="C4" s="13" t="s">
         <v>348</v>
-      </c>
-      <c r="C4" s="13" t="s">
-        <v>349</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B5" s="13" t="s">
+        <v>349</v>
+      </c>
+      <c r="C5" s="13" t="s">
         <v>350</v>
-      </c>
-      <c r="C5" s="13" t="s">
-        <v>351</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B6" s="13" t="s">
+        <v>351</v>
+      </c>
+      <c r="C6" s="16" t="s">
         <v>352</v>
-      </c>
-      <c r="C6" s="16" t="s">
-        <v>353</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>353</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>354</v>
-      </c>
-      <c r="C7" s="13" t="s">
-        <v>355</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B8" s="13" t="s">
+        <v>355</v>
+      </c>
+      <c r="C8" s="13" t="s">
         <v>356</v>
-      </c>
-      <c r="C8" s="13" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B9" s="16" t="s">
+        <v>357</v>
+      </c>
+      <c r="C9" s="13" t="s">
         <v>358</v>
-      </c>
-      <c r="C9" s="13" t="s">
-        <v>359</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B10" s="13" t="s">
+        <v>359</v>
+      </c>
+      <c r="C10" s="13" t="s">
         <v>360</v>
-      </c>
-      <c r="C10" s="13" t="s">
-        <v>361</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B11" s="13" t="s">
+        <v>361</v>
+      </c>
+      <c r="C11" s="13" t="s">
         <v>362</v>
-      </c>
-      <c r="C11" s="13" t="s">
-        <v>363</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B12" s="13" t="s">
+        <v>363</v>
+      </c>
+      <c r="C12" s="13" t="s">
         <v>364</v>
-      </c>
-      <c r="C12" s="13" t="s">
-        <v>365</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B13" s="13" t="s">
+        <v>365</v>
+      </c>
+      <c r="C13" s="13" t="s">
         <v>366</v>
-      </c>
-      <c r="C13" s="13" t="s">
-        <v>367</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B14" s="13" t="s">
+        <v>367</v>
+      </c>
+      <c r="C14" s="16" t="s">
         <v>368</v>
-      </c>
-      <c r="C14" s="16" t="s">
-        <v>369</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
       <c r="B15" s="13" t="s">
+        <v>369</v>
+      </c>
+      <c r="C15" s="13" t="s">
         <v>370</v>
-      </c>
-      <c r="C15" s="13" t="s">
-        <v>371</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
+        <v>371</v>
+      </c>
+      <c r="B16" s="16" t="s">
         <v>372</v>
       </c>
-      <c r="B16" s="16" t="s">
+      <c r="C16" s="13" t="s">
         <v>373</v>
-      </c>
-      <c r="C16" s="13" t="s">
-        <v>374</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B17" s="16" t="s">
+        <v>374</v>
+      </c>
+      <c r="C17" s="13" t="s">
         <v>375</v>
-      </c>
-      <c r="C17" s="13" t="s">
-        <v>376</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>377</v>
+        <v>376</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B19" s="13" t="s">
+        <v>377</v>
+      </c>
+      <c r="C19" s="13" t="s">
         <v>378</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>379</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>372</v>
+        <v>371</v>
       </c>
       <c r="B20" s="16" t="s">
+        <v>379</v>
+      </c>
+      <c r="C20" s="16" t="s">
         <v>380</v>
-      </c>
-      <c r="C20" s="16" t="s">
-        <v>381</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: reflect DX expected schedule (Nov test, Dec rollout)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Ev2GcePRwbwZKfH9HbtDvV
</commit_message>
<xml_diff>
--- a/docs/scrap-highlight/스크랩하이라이트_DS도입_관리.xlsx
+++ b/docs/scrap-highlight/스크랩하이라이트_DS도입_관리.xlsx
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="540" uniqueCount="381">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="546" uniqueCount="384">
   <si>
     <t xml:space="preserve">스크랩 하이라이트 DS 도입 — 과제 관리</t>
   </si>
@@ -158,7 +158,58 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">와 동일 시점 도입 </t>
+      <t xml:space="preserve">와 동일 시점 도입 — </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">예상</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: 11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 테스트 → </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 적용 </t>
     </r>
     <r>
       <rPr>
@@ -175,75 +226,16 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">김인철 상무 지시</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) · </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그룹 권고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">연내</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">적용</t>
+      <t xml:space="preserve">그룹 권고 일정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
     </r>
   </si>
   <si>
@@ -652,7 +644,7 @@
     <t xml:space="preserve">2026-10-28</t>
   </si>
   <si>
-    <t xml:space="preserve">이태양 프로·AX개발팀 모두 세부 일정 미확인(10.27 보고) → 김경수 파트장 통해 계속 확인</t>
+    <t xml:space="preserve">DX 예상: 11월 테스트, 12월 적용(그룹 권고 일정). 세부 일자는 추가 확인</t>
   </si>
   <si>
     <t xml:space="preserve">A3</t>
@@ -909,32 +901,32 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">일정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">' </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">시트</t>
+      <t xml:space="preserve">DX 11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 테스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 적용 기준으로 작성 가능</t>
     </r>
   </si>
   <si>
@@ -1819,7 +1811,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">DS </t>
+      <t xml:space="preserve">DX: </t>
     </r>
     <r>
       <rPr>
@@ -1828,7 +1820,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">목표 열을 채울 것 </t>
+      <t xml:space="preserve">그룹 권고 일정</t>
     </r>
     <r>
       <rPr>
@@ -1838,7 +1830,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">· </t>
+      <t xml:space="preserve">(11</t>
     </r>
     <r>
       <rPr>
@@ -1847,7 +1839,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">그룹 권고</t>
+      <t xml:space="preserve">월 테스트 → </t>
     </r>
     <r>
       <rPr>
@@ -1857,7 +1849,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">: 10</t>
+      <t xml:space="preserve">12</t>
     </r>
     <r>
       <rPr>
@@ -1866,7 +1858,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">월 착수 → </t>
+      <t xml:space="preserve">월 적용</t>
     </r>
     <r>
       <rPr>
@@ -1876,7 +1868,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">11</t>
+      <t xml:space="preserve">)</t>
     </r>
     <r>
       <rPr>
@@ -1885,7 +1877,7 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
-      <t xml:space="preserve">월 테스트 → </t>
+      <t xml:space="preserve">에 맞춰 진행 예정 </t>
     </r>
     <r>
       <rPr>
@@ -1895,7 +1887,7 @@
         <family val="0"/>
         <charset val="1"/>
       </rPr>
-      <t xml:space="preserve">12</t>
+      <t xml:space="preserve">· DS</t>
     </r>
     <r>
       <rPr>
@@ -1904,1121 +1896,1236 @@
         <rFont val="WenQuanYi Zen Hei"/>
         <family val="2"/>
       </rPr>
+      <t xml:space="preserve">도 동일 목표</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">단계</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그룹(참고)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DX</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS </t>
+    </r>
+    <r>
+      <rPr>
+        <b val="true"/>
+        <sz val="10"/>
+        <color rgb="FFFFFFFF"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">목표</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">선결</t>
+  </si>
+  <si>
+    <t xml:space="preserve">요청·샘플 전달</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">7.20 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">킥오프</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">10.12</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 말</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">A1, A3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">샘플 테스트·판정</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10.12 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">당일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">적용 가능</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">양식 맞춤 개발</t>
+  </si>
+  <si>
+    <t xml:space="preserve">7.20~8.27</t>
+  </si>
+  <si>
+    <t xml:space="preserve">불필요</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">A4 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">결과</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PC·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">계정</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보안 세팅</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">즉시 착수</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 테스트 전 완료</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">T3~T8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실운영 병행 테스트</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.27~9.12</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">본 적용</t>
+  </si>
+  <si>
+    <t xml:space="preserve">9.14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">12월</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(DX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">와 동일</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">관계자</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이름</t>
+  </si>
+  <si>
+    <t xml:space="preserve">직책·소속</t>
+  </si>
+  <si>
+    <t xml:space="preserve">역할</t>
+  </si>
+  <si>
+    <t xml:space="preserve">메일</t>
+  </si>
+  <si>
+    <t xml:space="preserve">연락 상태</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DS</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">컴팀장님</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">팀장</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공식 지원요청 메일 명의자</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김인철 (Jerome)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상무/그룹장</t>
+  </si>
+  <si>
+    <t xml:space="preserve">지시·팀장님 보고, 1일 2회 보고 수신</t>
+  </si>
+  <si>
+    <t xml:space="preserve">everpfe.kim@samsung.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이정섭 (Justin)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">파트장</t>
+  </si>
+  <si>
+    <t xml:space="preserve">진행 체크, 보고방 개설</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김인영 (Inyoung)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">진행 체크</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김기훈</t>
+  </si>
+  <si>
+    <t xml:space="preserve">부장</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김용호 프로 측 설명·조율</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이한정 (Cecilia)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실무 주도 / 08:00 보고</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실무 주도 / 18:00 보고, AX개발팀 실무방</t>
+  </si>
+  <si>
+    <t xml:space="preserve">그룹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">차병석</t>
+  </si>
+  <si>
+    <t xml:space="preserve">부사장/팀장 브랜드PR팀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">안내메일 발신, 백사장님 통합보고</t>
+  </si>
+  <si>
+    <t xml:space="preserve">bs.cha@samsung.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">박상권</t>
+  </si>
+  <si>
+    <t xml:space="preserve">통합보고 일정 전달</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김용호</t>
+  </si>
+  <si>
+    <t xml:space="preserve">프로 · 전자 PR기획그룹</t>
+  </si>
+  <si>
+    <t xml:space="preserve">사례 실무 문의 창구</t>
+  </si>
+  <si>
+    <t xml:space="preserve">yonghoc.kim@samsung.com</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10.26 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">통화</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">정홍욱</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상무/그룹장 국내미디어그룹</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">도입 책임</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">honguk.chung@samsung.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이태양</t>
+  </si>
+  <si>
+    <t xml:space="preserve">프로 국내미디어그룹</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">과제 실무</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">10.27 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메일 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">FW </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">받음</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">AX</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김경수</t>
+  </si>
+  <si>
+    <t xml:space="preserve">파트장 전사 AX개발팀 (우면동)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">기술 실무 핵심</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ks0326.kim@samsung.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">실무방</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이근택</t>
+  </si>
+  <si>
+    <t xml:space="preserve">프로 전사 AX개발팀</t>
+  </si>
+  <si>
+    <t xml:space="preserve">개발 실무</t>
+  </si>
+  <si>
+    <t xml:space="preserve">안재용</t>
+  </si>
+  <si>
+    <t xml:space="preserve">센터장 DX AX/PI센터</t>
+  </si>
+  <si>
+    <t xml:space="preserve">공식 지원요청 수신</t>
+  </si>
+  <si>
+    <t xml:space="preserve">미요청</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김상하</t>
+  </si>
+  <si>
+    <t xml:space="preserve">상무 DX AX/PI센터</t>
+  </si>
+  <si>
+    <t xml:space="preserve">경과 기록</t>
+  </si>
+  <si>
+    <t xml:space="preserve">새 사건은 맨 아래 행에 추가</t>
+  </si>
+  <si>
+    <t xml:space="preserve">일자</t>
+  </si>
+  <si>
+    <t xml:space="preserve">시각</t>
+  </si>
+  <si>
+    <t xml:space="preserve">주체</t>
+  </si>
+  <si>
+    <t xml:space="preserve">내용</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-06</t>
+  </si>
+  <si>
+    <t xml:space="preserve">홍보임원회의</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'AI </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">활용 스크랩 하이라이트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">' </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">언급</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-12</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10:57</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정홍욱 상무</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개발팀 김경수 파트장에 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">비즈니스</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">PR) </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">스크랩 적용 요청</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">샘플 전달</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">17:19</t>
+  </si>
+  <si>
+    <t xml:space="preserve">차병석 부사장</t>
+  </si>
+  <si>
+    <t xml:space="preserve">관계사 임원 대상 안내메일 발송 (권고: 10월 착수→11월 테스트→12월 적용)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">19:29</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김경수 파트장</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">샘플 테스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그룹과 양식</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">성능 유사</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">. </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">특이 편집 기사 미적용</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">(</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">학습 시 샘플 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">50+)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">2026-10-13</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:15</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김인철 상무</t>
+  </si>
+  <si>
+    <t xml:space="preserve">안내메일 FW: '팀장님께서는 양진호, 이한정님에게 맡길 요량'. 이한정 수신 누락, 구두 지시 없음</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">특이 편집 기사 추가 학습 불필요</t>
+  </si>
+  <si>
+    <t xml:space="preserve">팀장님</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이한정에게 전화: '전사 AX 과제 왜 안 하고 있어?'</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:11</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DS</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">만 피드백 없음 지적</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">17:14</t>
+  </si>
+  <si>
+    <t xml:space="preserve">담당 지정: 양진호·이한정. 오늘 중 김용호 연락. '제 불찰'로 팀장님께 보고</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:18</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이정섭 파트장</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보고방 개설</t>
+  </si>
+  <si>
+    <t xml:space="preserve">오늘 중 김용호 컨택, 수시 보고, 팀장님 보고용 정리</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:38</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">1</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">차 보고</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">김용호 통화</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, DX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">는 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">AX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">개발팀과 진행 중</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, DS </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">양식 맞춤 개발</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">·</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">테스트 필요</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">이태양 연락</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">17:44</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">와 가능하면 동일 시점 도입 지시</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">17:45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">매일 08:00 이한정 / 18:00 양진호 보고, 텔레그램 전환 지시</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:46</t>
+  </si>
+  <si>
+    <t xml:space="preserve">차병석 부사장 → 백사장님 각 사별 통합 보고 예정</t>
+  </si>
+  <si>
+    <t xml:space="preserve">김기훈 부장: 김용호 측 잘 설명</t>
+  </si>
+  <si>
+    <t xml:space="preserve">17:49</t>
+  </si>
+  <si>
+    <t xml:space="preserve">필요하면 직접 찾아가 만날 것</t>
+  </si>
+  <si>
+    <t xml:space="preserve">07:43</t>
+  </si>
+  <si>
+    <t xml:space="preserve">이태양 프로</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">메일스레드 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">FW (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">선행조건 안내 포함</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">08:01</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">'?' (</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">보고 재촉</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">)</t>
+    </r>
+  </si>
+  <si>
+    <t xml:space="preserve">08:03</t>
+  </si>
+  <si>
+    <t xml:space="preserve">정기 보고: 팀장님 명의 공식 요청 필요, AX개발팀 실무방 개설, DX 도입일 미정(개발팀도 미확인), DS 보안 절차 확인 필요</t>
+  </si>
+  <si>
+    <t xml:space="preserve">09:11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보고 가이드: 오전=당일 진행계획, 오후=당일 진행결과. 둘을 무 자르듯 분리(재방송 방지), 08:00은 전날 작성 후 예약 발신</t>
+  </si>
+  <si>
+    <t xml:space="preserve">보고방 텔레그램 전환 완료</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">DX </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">예상 일정 확인</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">: </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">그룹 권고 일정에 맞춰 </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">11</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve">월 테스트</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="맑은 고딕"/>
+        <family val="0"/>
+        <charset val="1"/>
+      </rPr>
+      <t xml:space="preserve">, 12</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="10"/>
+        <rFont val="WenQuanYi Zen Hei"/>
+        <family val="2"/>
+      </rPr>
       <t xml:space="preserve">월 적용</t>
     </r>
-  </si>
-  <si>
-    <t xml:space="preserve">단계</t>
-  </si>
-  <si>
-    <t xml:space="preserve">그룹(참고)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DX</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS </t>
-    </r>
-    <r>
-      <rPr>
-        <b val="true"/>
-        <sz val="10"/>
-        <color rgb="FFFFFFFF"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">목표</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">선결</t>
-  </si>
-  <si>
-    <t xml:space="preserve">요청·샘플 전달</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">7.20 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">킥오프</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">10.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">A1, A3</t>
-  </si>
-  <si>
-    <t xml:space="preserve">샘플 테스트·판정</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10.12 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">당일 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">적용 가능</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">양식 맞춤 개발</t>
-  </si>
-  <si>
-    <t xml:space="preserve">7.20~8.27</t>
-  </si>
-  <si>
-    <t xml:space="preserve">불필요</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">A4 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">결과</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">PC·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">계정</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보안 세팅</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">T3~T8</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실운영 병행 테스트</t>
-  </si>
-  <si>
-    <t xml:space="preserve">8.27~9.12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">?</t>
-  </si>
-  <si>
-    <t xml:space="preserve">본 적용</t>
-  </si>
-  <si>
-    <t xml:space="preserve">9.14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미정</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도입일과 동일 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">늦어도 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">12</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">월</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">관계자</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이름</t>
-  </si>
-  <si>
-    <t xml:space="preserve">직책·소속</t>
-  </si>
-  <si>
-    <t xml:space="preserve">역할</t>
-  </si>
-  <si>
-    <t xml:space="preserve">메일</t>
-  </si>
-  <si>
-    <t xml:space="preserve">연락 상태</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DS</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">컴팀장님</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">팀장</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공식 지원요청 메일 명의자</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김인철 (Jerome)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">상무/그룹장</t>
-  </si>
-  <si>
-    <t xml:space="preserve">지시·팀장님 보고, 1일 2회 보고 수신</t>
-  </si>
-  <si>
-    <t xml:space="preserve">everpfe.kim@samsung.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이정섭 (Justin)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">파트장</t>
-  </si>
-  <si>
-    <t xml:space="preserve">진행 체크, 보고방 개설</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김인영 (Inyoung)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">진행 체크</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김기훈</t>
-  </si>
-  <si>
-    <t xml:space="preserve">부장</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김용호 프로 측 설명·조율</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이한정 (Cecilia)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실무 주도 / 08:00 보고</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실무 주도 / 18:00 보고, AX개발팀 실무방</t>
-  </si>
-  <si>
-    <t xml:space="preserve">그룹</t>
-  </si>
-  <si>
-    <t xml:space="preserve">차병석</t>
-  </si>
-  <si>
-    <t xml:space="preserve">부사장/팀장 브랜드PR팀</t>
-  </si>
-  <si>
-    <t xml:space="preserve">안내메일 발신, 백사장님 통합보고</t>
-  </si>
-  <si>
-    <t xml:space="preserve">bs.cha@samsung.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">박상권</t>
-  </si>
-  <si>
-    <t xml:space="preserve">통합보고 일정 전달</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김용호</t>
-  </si>
-  <si>
-    <t xml:space="preserve">프로 · 전자 PR기획그룹</t>
-  </si>
-  <si>
-    <t xml:space="preserve">사례 실무 문의 창구</t>
-  </si>
-  <si>
-    <t xml:space="preserve">yonghoc.kim@samsung.com</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10.26 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">통화</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">정홍욱</t>
-  </si>
-  <si>
-    <t xml:space="preserve">상무/그룹장 국내미디어그룹</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">도입 책임</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">honguk.chung@samsung.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이태양</t>
-  </si>
-  <si>
-    <t xml:space="preserve">프로 국내미디어그룹</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">과제 실무</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">10.27 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">메일 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FW </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">받음</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">AX</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김경수</t>
-  </si>
-  <si>
-    <t xml:space="preserve">파트장 전사 AX개발팀 (우면동)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">기술 실무 핵심</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ks0326.kim@samsung.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">실무방</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이근택</t>
-  </si>
-  <si>
-    <t xml:space="preserve">프로 전사 AX개발팀</t>
-  </si>
-  <si>
-    <t xml:space="preserve">개발 실무</t>
-  </si>
-  <si>
-    <t xml:space="preserve">안재용</t>
-  </si>
-  <si>
-    <t xml:space="preserve">센터장 DX AX/PI센터</t>
-  </si>
-  <si>
-    <t xml:space="preserve">공식 지원요청 수신</t>
-  </si>
-  <si>
-    <t xml:space="preserve">미요청</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김상하</t>
-  </si>
-  <si>
-    <t xml:space="preserve">상무 DX AX/PI센터</t>
-  </si>
-  <si>
-    <t xml:space="preserve">경과 기록</t>
-  </si>
-  <si>
-    <t xml:space="preserve">새 사건은 맨 아래 행에 추가</t>
-  </si>
-  <si>
-    <t xml:space="preserve">일자</t>
-  </si>
-  <si>
-    <t xml:space="preserve">시각</t>
-  </si>
-  <si>
-    <t xml:space="preserve">주체</t>
-  </si>
-  <si>
-    <t xml:space="preserve">내용</t>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-06</t>
-  </si>
-  <si>
-    <t xml:space="preserve">홍보임원회의</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'AI </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">활용 스크랩 하이라이트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">' </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">언급</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-12</t>
-  </si>
-  <si>
-    <t xml:space="preserve">10:57</t>
-  </si>
-  <si>
-    <t xml:space="preserve">정홍욱 상무</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개발팀 김경수 파트장에 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">비즈니스</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">PR) </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">스크랩 적용 요청</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">샘플 전달</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">17:19</t>
-  </si>
-  <si>
-    <t xml:space="preserve">차병석 부사장</t>
-  </si>
-  <si>
-    <t xml:space="preserve">관계사 임원 대상 안내메일 발송 (권고: 10월 착수→11월 테스트→12월 적용)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">19:29</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김경수 파트장</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">샘플 테스트</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">그룹과 양식</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">성능 유사</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">. </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">특이 편집 기사 미적용</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">(</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">학습 시 샘플 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">50+)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">2026-10-13</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07:15</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김인철 상무</t>
-  </si>
-  <si>
-    <t xml:space="preserve">안내메일 FW: '팀장님께서는 양진호, 이한정님에게 맡길 요량'. 이한정 수신 누락, 구두 지시 없음</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07:18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">특이 편집 기사 추가 학습 불필요</t>
-  </si>
-  <si>
-    <t xml:space="preserve">팀장님</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이한정에게 전화: '전사 AX 과제 왜 안 하고 있어?'</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:11</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DS</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">만 피드백 없음 지적</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">17:14</t>
-  </si>
-  <si>
-    <t xml:space="preserve">담당 지정: 양진호·이한정. 오늘 중 김용호 연락. '제 불찰'로 팀장님께 보고</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:18</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이정섭 파트장</t>
-  </si>
-  <si>
-    <t xml:space="preserve">보고방 개설</t>
-  </si>
-  <si>
-    <t xml:space="preserve">오늘 중 김용호 컨택, 수시 보고, 팀장님 보고용 정리</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:38</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">1</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">차 보고</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">: </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">김용호 통화</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, DX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">는 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">AX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">개발팀과 진행 중</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, DS </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">양식 맞춤 개발</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">·</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">테스트 필요</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">, </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">이태양 연락</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">17:44</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">와 가능하면 동일 시점 도입 지시</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">17:45</t>
-  </si>
-  <si>
-    <t xml:space="preserve">매일 08:00 이한정 / 18:00 양진호 보고, 텔레그램 전환 지시</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:46</t>
-  </si>
-  <si>
-    <t xml:space="preserve">차병석 부사장 → 백사장님 각 사별 통합 보고 예정</t>
-  </si>
-  <si>
-    <t xml:space="preserve">김기훈 부장: 김용호 측 잘 설명</t>
-  </si>
-  <si>
-    <t xml:space="preserve">17:49</t>
-  </si>
-  <si>
-    <t xml:space="preserve">필요하면 직접 찾아가 만날 것</t>
-  </si>
-  <si>
-    <t xml:space="preserve">07:43</t>
-  </si>
-  <si>
-    <t xml:space="preserve">이태양 프로</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">DX </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">메일스레드 </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">FW (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">선행조건 안내 포함</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">08:01</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">'?' (</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="WenQuanYi Zen Hei"/>
-        <family val="2"/>
-      </rPr>
-      <t xml:space="preserve">보고 재촉</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="10"/>
-        <rFont val="맑은 고딕"/>
-        <family val="0"/>
-        <charset val="1"/>
-      </rPr>
-      <t xml:space="preserve">)</t>
-    </r>
-  </si>
-  <si>
-    <t xml:space="preserve">08:03</t>
-  </si>
-  <si>
-    <t xml:space="preserve">정기 보고: 팀장님 명의 공식 요청 필요, AX개발팀 실무방 개설, DX 도입일 미정(개발팀도 미확인), DS 보안 절차 확인 필요</t>
-  </si>
-  <si>
-    <t xml:space="preserve">09:11</t>
-  </si>
-  <si>
-    <t xml:space="preserve">보고 가이드: 오전=당일 진행계획, 오후=당일 진행결과. 둘을 무 자르듯 분리(재방송 방지), 08:00은 전날 작성 후 예약 발신</t>
-  </si>
-  <si>
-    <t xml:space="preserve">보고방 텔레그램 전환 완료</t>
   </si>
   <si>
     <t xml:space="preserve">정기 보고</t>
@@ -6687,7 +6794,7 @@
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="9" fillId="0" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="9" fillId="4" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="true" applyProtection="false">
       <alignment horizontal="general" vertical="top" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -8056,9 +8163,11 @@
       <c r="C5" s="16" t="s">
         <v>168</v>
       </c>
-      <c r="D5" s="20"/>
+      <c r="D5" s="20" t="s">
+        <v>169</v>
+      </c>
       <c r="E5" s="16" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="F5" s="13" t="s">
         <v>18</v>
@@ -8066,13 +8175,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B6" s="16" t="s">
         <v>95</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="D6" s="20"/>
       <c r="E6" s="16" t="s">
@@ -8084,17 +8193,17 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="D7" s="20"/>
       <c r="E7" s="16" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="F7" s="13" t="s">
         <v>18</v>
@@ -8102,7 +8211,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B8" s="16" t="s">
         <v>95</v>
@@ -8110,9 +8219,11 @@
       <c r="C8" s="13" t="s">
         <v>19</v>
       </c>
-      <c r="D8" s="20"/>
+      <c r="D8" s="21" t="s">
+        <v>178</v>
+      </c>
       <c r="E8" s="16" t="s">
-        <v>177</v>
+        <v>179</v>
       </c>
       <c r="F8" s="13" t="s">
         <v>18</v>
@@ -8120,15 +8231,17 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>178</v>
+        <v>180</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>179</v>
+        <v>181</v>
       </c>
       <c r="C9" s="16" t="s">
-        <v>180</v>
-      </c>
-      <c r="D9" s="20"/>
+        <v>182</v>
+      </c>
+      <c r="D9" s="20" t="s">
+        <v>182</v>
+      </c>
       <c r="E9" s="16" t="s">
         <v>101</v>
       </c>
@@ -8138,16 +8251,16 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>181</v>
+        <v>183</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>182</v>
+        <v>184</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>183</v>
+        <v>185</v>
       </c>
       <c r="D10" s="20" t="s">
-        <v>184</v>
+        <v>186</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="13" t="s">
@@ -8203,7 +8316,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8211,181 +8324,181 @@
         <v>17</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
       <c r="D3" s="19" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="E3" s="19" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
       <c r="F3" s="19" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B4" s="16" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>193</v>
+        <v>195</v>
       </c>
       <c r="D4" s="13" t="s">
-        <v>194</v>
+        <v>196</v>
       </c>
       <c r="E4" s="16"/>
       <c r="F4" s="16"/>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>197</v>
+        <v>199</v>
       </c>
       <c r="E5" s="16" t="s">
-        <v>198</v>
+        <v>200</v>
       </c>
       <c r="F5" s="16"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>199</v>
+        <v>201</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>200</v>
+        <v>202</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>201</v>
+        <v>203</v>
       </c>
       <c r="E6" s="16"/>
       <c r="F6" s="16"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B7" s="13" t="s">
+        <v>204</v>
+      </c>
+      <c r="C7" s="13" t="s">
         <v>202</v>
       </c>
-      <c r="C7" s="13" t="s">
-        <v>200</v>
-      </c>
       <c r="D7" s="13" t="s">
-        <v>203</v>
+        <v>205</v>
       </c>
       <c r="E7" s="16"/>
       <c r="F7" s="16"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>204</v>
+        <v>206</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="E8" s="16"/>
       <c r="F8" s="16"/>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B9" s="13" t="s">
-        <v>207</v>
+        <v>209</v>
       </c>
       <c r="C9" s="16"/>
       <c r="D9" s="13" t="s">
-        <v>208</v>
+        <v>210</v>
       </c>
       <c r="E9" s="16"/>
       <c r="F9" s="16"/>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>191</v>
+        <v>193</v>
       </c>
       <c r="B10" s="13" t="s">
         <v>72</v>
       </c>
       <c r="C10" s="16"/>
       <c r="D10" s="13" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="E10" s="16"/>
       <c r="F10" s="16"/>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>211</v>
+        <v>213</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>212</v>
+        <v>214</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>213</v>
+        <v>215</v>
       </c>
       <c r="E11" s="16" t="s">
-        <v>214</v>
+        <v>216</v>
       </c>
       <c r="F11" s="16"/>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="C12" s="16"/>
       <c r="D12" s="13" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="E12" s="16"/>
       <c r="F12" s="16"/>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>210</v>
+        <v>212</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>217</v>
+        <v>219</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="E13" s="16" t="s">
-        <v>220</v>
+        <v>222</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>221</v>
+        <v>223</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8393,16 +8506,16 @@
         <v>163</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D14" s="16" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="E14" s="16" t="s">
-        <v>225</v>
+        <v>227</v>
       </c>
       <c r="F14" s="16"/>
     </row>
@@ -8411,91 +8524,91 @@
         <v>163</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>226</v>
+        <v>228</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>227</v>
+        <v>229</v>
       </c>
       <c r="D15" s="16" t="s">
-        <v>228</v>
+        <v>230</v>
       </c>
       <c r="E15" s="16"/>
       <c r="F15" s="16" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B16" s="13" t="s">
-        <v>231</v>
+        <v>233</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>232</v>
+        <v>234</v>
       </c>
       <c r="D16" s="13" t="s">
-        <v>233</v>
+        <v>235</v>
       </c>
       <c r="E16" s="16" t="s">
-        <v>234</v>
+        <v>236</v>
       </c>
       <c r="F16" s="13" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B17" s="13" t="s">
-        <v>236</v>
+        <v>238</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>237</v>
+        <v>239</v>
       </c>
       <c r="D17" s="13" t="s">
-        <v>238</v>
+        <v>240</v>
       </c>
       <c r="E17" s="16"/>
       <c r="F17" s="13" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B18" s="13" t="s">
-        <v>239</v>
+        <v>241</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>240</v>
+        <v>242</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="E18" s="16"/>
       <c r="F18" s="13" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>230</v>
+        <v>232</v>
       </c>
       <c r="B19" s="13" t="s">
+        <v>245</v>
+      </c>
+      <c r="C19" s="13" t="s">
+        <v>246</v>
+      </c>
+      <c r="D19" s="13" t="s">
         <v>243</v>
-      </c>
-      <c r="C19" s="13" t="s">
-        <v>244</v>
-      </c>
-      <c r="D19" s="13" t="s">
-        <v>241</v>
       </c>
       <c r="E19" s="16"/>
       <c r="F19" s="13" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
     </row>
   </sheetData>
@@ -8514,7 +8627,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="1" width="12"/>
@@ -8525,108 +8638,108 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>245</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="19" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B4" s="19" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C4" s="19" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D4" s="19" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="16" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="B5" s="16"/>
       <c r="C5" s="13" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="D5" s="16" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D6" s="16" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B7" s="16" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="16" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="B8" s="16" t="s">
-        <v>261</v>
+        <v>263</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>262</v>
+        <v>264</v>
       </c>
       <c r="D8" s="16" t="s">
-        <v>263</v>
+        <v>265</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="16" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>265</v>
+        <v>267</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D9" s="13" t="s">
-        <v>267</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="16" t="s">
-        <v>264</v>
+        <v>266</v>
       </c>
       <c r="B10" s="16" t="s">
-        <v>268</v>
+        <v>270</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="D10" s="13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8635,10 +8748,10 @@
       </c>
       <c r="B11" s="16"/>
       <c r="C11" s="13" t="s">
-        <v>270</v>
+        <v>272</v>
       </c>
       <c r="D11" s="13" t="s">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8646,13 +8759,13 @@
         <v>107</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>272</v>
+        <v>274</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D12" s="16" t="s">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8660,13 +8773,13 @@
         <v>107</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>274</v>
+        <v>276</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D13" s="13" t="s">
-        <v>275</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8674,13 +8787,13 @@
         <v>107</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>276</v>
+        <v>278</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>277</v>
+        <v>279</v>
       </c>
       <c r="D14" s="13" t="s">
-        <v>278</v>
+        <v>280</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8688,13 +8801,13 @@
         <v>107</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D15" s="13" t="s">
-        <v>279</v>
+        <v>281</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8702,13 +8815,13 @@
         <v>107</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>280</v>
+        <v>282</v>
       </c>
       <c r="C16" s="13" t="s">
         <v>66</v>
       </c>
       <c r="D16" s="16" t="s">
-        <v>281</v>
+        <v>283</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8716,13 +8829,13 @@
         <v>107</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>282</v>
+        <v>284</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D17" s="16" t="s">
-        <v>283</v>
+        <v>285</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8730,13 +8843,13 @@
         <v>107</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D18" s="13" t="s">
-        <v>285</v>
+        <v>287</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8744,13 +8857,13 @@
         <v>107</v>
       </c>
       <c r="B19" s="16" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>215</v>
+        <v>217</v>
       </c>
       <c r="D19" s="13" t="s">
-        <v>287</v>
+        <v>289</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8758,13 +8871,13 @@
         <v>107</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>286</v>
+        <v>288</v>
       </c>
       <c r="C20" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D20" s="13" t="s">
-        <v>288</v>
+        <v>290</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8772,13 +8885,13 @@
         <v>107</v>
       </c>
       <c r="B21" s="16" t="s">
-        <v>289</v>
+        <v>291</v>
       </c>
       <c r="C21" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D21" s="13" t="s">
-        <v>290</v>
+        <v>292</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8786,13 +8899,13 @@
         <v>61</v>
       </c>
       <c r="B22" s="16" t="s">
-        <v>291</v>
+        <v>293</v>
       </c>
       <c r="C22" s="13" t="s">
-        <v>292</v>
+        <v>294</v>
       </c>
       <c r="D22" s="16" t="s">
-        <v>293</v>
+        <v>295</v>
       </c>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8800,13 +8913,13 @@
         <v>61</v>
       </c>
       <c r="B23" s="16" t="s">
-        <v>294</v>
+        <v>296</v>
       </c>
       <c r="C23" s="13" t="s">
-        <v>266</v>
+        <v>268</v>
       </c>
       <c r="D23" s="16" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8814,13 +8927,13 @@
         <v>61</v>
       </c>
       <c r="B24" s="16" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C24" s="13" t="s">
         <v>66</v>
       </c>
       <c r="D24" s="13" t="s">
-        <v>297</v>
+        <v>299</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -8828,16 +8941,16 @@
         <v>61</v>
       </c>
       <c r="B25" s="16" t="s">
-        <v>298</v>
+        <v>300</v>
       </c>
       <c r="C25" s="13" t="s">
         <v>99</v>
       </c>
       <c r="D25" s="13" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A26" s="16" t="s">
         <v>61</v>
       </c>
@@ -8845,8 +8958,20 @@
       <c r="C26" s="16" t="s">
         <v>95</v>
       </c>
-      <c r="D26" s="21" t="s">
-        <v>300</v>
+      <c r="D26" s="13" t="s">
+        <v>302</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="16" t="s">
+        <v>61</v>
+      </c>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16" t="s">
+        <v>95</v>
+      </c>
+      <c r="D27" s="16" t="s">
+        <v>303</v>
       </c>
     </row>
   </sheetData>
@@ -8878,17 +9003,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>301</v>
+        <v>304</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>302</v>
+        <v>305</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="11" t="s">
-        <v>303</v>
+        <v>306</v>
       </c>
       <c r="B4" s="22"/>
       <c r="C4" s="22"/>
@@ -8901,7 +9026,7 @@
         <v>17</v>
       </c>
       <c r="B5" s="14" t="s">
-        <v>304</v>
+        <v>307</v>
       </c>
       <c r="C5" s="14"/>
       <c r="D5" s="14"/>
@@ -8910,10 +9035,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="24" t="s">
-        <v>305</v>
+        <v>308</v>
       </c>
       <c r="B6" s="14" t="s">
-        <v>306</v>
+        <v>309</v>
       </c>
       <c r="C6" s="14"/>
       <c r="D6" s="14"/>
@@ -8922,10 +9047,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="24" t="s">
-        <v>307</v>
+        <v>310</v>
       </c>
       <c r="B7" s="14" t="s">
-        <v>308</v>
+        <v>311</v>
       </c>
       <c r="C7" s="14"/>
       <c r="D7" s="14"/>
@@ -8934,10 +9059,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="23" t="s">
-        <v>309</v>
+        <v>312</v>
       </c>
       <c r="B8" s="15" t="s">
-        <v>310</v>
+        <v>313</v>
       </c>
       <c r="C8" s="15"/>
       <c r="D8" s="15"/>
@@ -8946,10 +9071,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="23" t="s">
-        <v>311</v>
+        <v>314</v>
       </c>
       <c r="B9" s="14" t="s">
-        <v>312</v>
+        <v>315</v>
       </c>
       <c r="C9" s="14"/>
       <c r="D9" s="14"/>
@@ -8958,62 +9083,62 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="11" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="C11" s="11" t="s">
-        <v>313</v>
+        <v>316</v>
       </c>
       <c r="D11" s="11" t="s">
-        <v>314</v>
+        <v>317</v>
       </c>
       <c r="E11" s="11" t="s">
-        <v>315</v>
+        <v>318</v>
       </c>
       <c r="F11" s="11" t="s">
-        <v>316</v>
+        <v>319</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B12" s="16" t="s">
-        <v>318</v>
+        <v>321</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>319</v>
+        <v>322</v>
       </c>
       <c r="D12" s="13" t="s">
         <v>66</v>
       </c>
       <c r="E12" s="13" t="s">
-        <v>320</v>
+        <v>323</v>
       </c>
       <c r="F12" s="16" t="s">
-        <v>321</v>
+        <v>324</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>317</v>
+        <v>320</v>
       </c>
       <c r="B13" s="16" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D13" s="13" t="s">
         <v>72</v>
       </c>
       <c r="E13" s="13" t="s">
-        <v>324</v>
+        <v>327</v>
       </c>
       <c r="F13" s="16" t="s">
-        <v>325</v>
+        <v>328</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="408.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9021,19 +9146,19 @@
         <v>61</v>
       </c>
       <c r="B14" s="16" t="s">
-        <v>296</v>
+        <v>298</v>
       </c>
       <c r="C14" s="13" t="s">
-        <v>326</v>
+        <v>329</v>
       </c>
       <c r="D14" s="13" t="s">
         <v>66</v>
       </c>
       <c r="E14" s="13" t="s">
-        <v>327</v>
+        <v>330</v>
       </c>
       <c r="F14" s="16" t="s">
-        <v>328</v>
+        <v>331</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="300" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -9041,19 +9166,19 @@
         <v>61</v>
       </c>
       <c r="B15" s="16" t="s">
-        <v>322</v>
+        <v>325</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>323</v>
+        <v>326</v>
       </c>
       <c r="D15" s="13" t="s">
         <v>72</v>
       </c>
       <c r="E15" s="20" t="s">
-        <v>329</v>
+        <v>332</v>
       </c>
       <c r="F15" s="20" t="s">
-        <v>330</v>
+        <v>333</v>
       </c>
     </row>
   </sheetData>
@@ -9089,52 +9214,52 @@
   <sheetData>
     <row r="1" customFormat="false" ht="18.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="25" t="s">
-        <v>331</v>
+        <v>334</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="17" t="s">
-        <v>332</v>
+        <v>335</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="26" t="s">
-        <v>333</v>
+        <v>336</v>
       </c>
       <c r="B4" s="20" t="s">
-        <v>334</v>
+        <v>337</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="26" t="s">
-        <v>335</v>
+        <v>338</v>
       </c>
       <c r="B5" s="16" t="s">
-        <v>336</v>
+        <v>339</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="26" t="s">
-        <v>337</v>
+        <v>340</v>
       </c>
       <c r="B6" s="16" t="s">
-        <v>338</v>
+        <v>341</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="26" t="s">
-        <v>339</v>
+        <v>342</v>
       </c>
       <c r="B7" s="20" t="s">
-        <v>340</v>
+        <v>343</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="420" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="26" t="s">
-        <v>341</v>
+        <v>344</v>
       </c>
       <c r="B8" s="27" t="s">
-        <v>342</v>
+        <v>345</v>
       </c>
     </row>
   </sheetData>
@@ -9163,205 +9288,205 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A1" s="2" t="s">
-        <v>343</v>
+        <v>346</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A3" s="19" t="s">
-        <v>344</v>
+        <v>347</v>
       </c>
       <c r="B3" s="19" t="s">
-        <v>345</v>
+        <v>348</v>
       </c>
       <c r="C3" s="19" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A4" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B4" s="13" t="s">
-        <v>347</v>
+        <v>350</v>
       </c>
       <c r="C4" s="13" t="s">
-        <v>348</v>
+        <v>351</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A5" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B5" s="13" t="s">
-        <v>349</v>
+        <v>352</v>
       </c>
       <c r="C5" s="13" t="s">
-        <v>350</v>
+        <v>353</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A6" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B6" s="13" t="s">
-        <v>351</v>
+        <v>354</v>
       </c>
       <c r="C6" s="16" t="s">
-        <v>352</v>
+        <v>355</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A7" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B7" s="13" t="s">
-        <v>353</v>
+        <v>356</v>
       </c>
       <c r="C7" s="13" t="s">
-        <v>354</v>
+        <v>357</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B8" s="13" t="s">
-        <v>355</v>
+        <v>358</v>
       </c>
       <c r="C8" s="13" t="s">
-        <v>356</v>
+        <v>359</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A9" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B9" s="16" t="s">
-        <v>357</v>
+        <v>360</v>
       </c>
       <c r="C9" s="13" t="s">
-        <v>358</v>
+        <v>361</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A10" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B10" s="13" t="s">
-        <v>359</v>
+        <v>362</v>
       </c>
       <c r="C10" s="13" t="s">
-        <v>360</v>
+        <v>363</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A11" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B11" s="13" t="s">
-        <v>361</v>
+        <v>364</v>
       </c>
       <c r="C11" s="13" t="s">
-        <v>362</v>
+        <v>365</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A12" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B12" s="13" t="s">
-        <v>363</v>
+        <v>366</v>
       </c>
       <c r="C12" s="13" t="s">
-        <v>364</v>
+        <v>367</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B13" s="13" t="s">
-        <v>365</v>
+        <v>368</v>
       </c>
       <c r="C13" s="13" t="s">
-        <v>366</v>
+        <v>369</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B14" s="13" t="s">
-        <v>367</v>
+        <v>370</v>
       </c>
       <c r="C14" s="16" t="s">
-        <v>368</v>
+        <v>371</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>346</v>
+        <v>349</v>
       </c>
       <c r="B15" s="13" t="s">
-        <v>369</v>
+        <v>372</v>
       </c>
       <c r="C15" s="13" t="s">
-        <v>370</v>
+        <v>373</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A16" s="16" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B16" s="16" t="s">
-        <v>372</v>
+        <v>375</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>373</v>
+        <v>376</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A17" s="16" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B17" s="16" t="s">
-        <v>374</v>
+        <v>377</v>
       </c>
       <c r="C17" s="13" t="s">
-        <v>375</v>
+        <v>378</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A18" s="16" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B18" s="16" t="s">
-        <v>376</v>
+        <v>379</v>
       </c>
       <c r="C18" s="13" t="s">
-        <v>269</v>
+        <v>271</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="26.25" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A19" s="16" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>377</v>
+        <v>380</v>
       </c>
       <c r="C19" s="13" t="s">
-        <v>378</v>
+        <v>381</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A20" s="16" t="s">
-        <v>371</v>
+        <v>374</v>
       </c>
       <c r="B20" s="16" t="s">
-        <v>379</v>
+        <v>382</v>
       </c>
       <c r="C20" s="16" t="s">
-        <v>380</v>
+        <v>383</v>
       </c>
     </row>
   </sheetData>

</xml_diff>